<commit_message>
Update 2025 MLS projections for CMM 24-06
</commit_message>
<xml_diff>
--- a/2025-MLS-projections/BSIA Catch/2021-2024 BSIA MLS Catch.xlsx
+++ b/2025-MLS-projections/BSIA Catch/2021-2024 BSIA MLS Catch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jon.brodziak\Desktop\2024 WCNPO MLS Rebuilding\2025 MLS projections\BSIA Catch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA5B72A3-DD65-4244-AC47-28A93552B48A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81961F3B-ACFB-4A6E-93B6-689BB6A2BD4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="16663" windowHeight="8863" firstSheet="1" activeTab="3" xr2:uid="{416E3EAD-1861-4C87-937B-DDBEC44D9B39}"/>
   </bookViews>
@@ -36,8 +36,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="29">
   <si>
     <t>G3</t>
   </si>
@@ -115,6 +137,15 @@
   </si>
   <si>
     <t>Total BSIA for WCNPO MLS Catch Biomass by Fleet Group</t>
+  </si>
+  <si>
+    <t>Observed</t>
+  </si>
+  <si>
+    <t>F-Based</t>
+  </si>
+  <si>
+    <t>% Change</t>
   </si>
 </sst>
 </file>
@@ -124,7 +155,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -141,6 +172,13 @@
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -333,10 +371,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -345,15 +384,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -423,9 +453,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -454,12 +481,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -470,9 +491,58 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1244,7 +1314,7 @@
     <col min="7" max="7" width="4.69140625" customWidth="1"/>
     <col min="8" max="8" width="7" customWidth="1"/>
     <col min="9" max="9" width="9.53515625" customWidth="1"/>
-    <col min="10" max="10" width="7.23046875" customWidth="1"/>
+    <col min="10" max="10" width="9.4609375" customWidth="1"/>
     <col min="11" max="11" width="10.61328125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6.84375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="2.69140625" customWidth="1"/>
@@ -1257,257 +1327,337 @@
     <col min="26" max="26" width="7.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="20.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:11" ht="20.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4"/>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="8"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="45"/>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="7">
         <v>2021</v>
       </c>
-      <c r="C4" s="11">
+      <c r="C4" s="8">
         <v>2022</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="8">
         <v>2023</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="9">
         <v>2024</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A5" s="28" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A5" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="12">
         <v>118.18600000000001</v>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="13">
         <v>74.753</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="13">
         <v>128.80199999999999</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="13">
         <v>82.938999999999993</v>
       </c>
-      <c r="F5" s="17">
+      <c r="F5" s="14">
         <f>AVERAGE(B5:E5)</f>
         <v>101.16999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A6" s="29" t="s">
+    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="18">
+      <c r="B6" s="15">
         <v>100.309</v>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="16">
         <v>98.667000000000002</v>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="16">
         <v>80.421000000000006</v>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="16">
         <v>176.49799999999999</v>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="17">
         <f t="shared" ref="F6:F13" si="0">AVERAGE(B6:E6)</f>
         <v>113.97375</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A7" s="29" t="s">
+    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="15">
         <v>551.13499999999999</v>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="16">
         <v>464.16500000000002</v>
       </c>
-      <c r="D7" s="19">
+      <c r="D7" s="16">
         <v>525.50099999999998</v>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="16">
         <v>577.67599999999993</v>
       </c>
-      <c r="F7" s="20">
+      <c r="F7" s="17">
         <f t="shared" si="0"/>
         <v>529.61924999999997</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A8" s="29" t="s">
+      <c r="H7" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" s="53" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A8" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="15">
         <v>71.613</v>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="16">
         <v>36.423000000000002</v>
       </c>
-      <c r="D8" s="19">
+      <c r="D8" s="16">
         <v>27.530999999999999</v>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="16">
         <v>26.783999999999999</v>
       </c>
-      <c r="F8" s="20">
+      <c r="F8" s="17">
         <f t="shared" si="0"/>
         <v>40.58775</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A9" s="29" t="s">
+      <c r="H8" s="54">
+        <v>2021</v>
+      </c>
+      <c r="I8" s="49" cm="1">
+        <f t="array" ref="I8:I11">TRANSPOSE(B14:E14)</f>
+        <v>1539.7965823166828</v>
+      </c>
+      <c r="J8" s="29">
+        <v>2910</v>
+      </c>
+      <c r="K8" s="50">
+        <f>(I8-J8)/J8</f>
+        <v>-0.47086028099083066</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A9" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="18">
+      <c r="B9" s="15">
         <v>89.24</v>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="16">
         <v>79.738</v>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="16">
         <v>110.13000000000001</v>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="16">
         <v>110.13000000000001</v>
       </c>
-      <c r="F9" s="20">
+      <c r="F9" s="17">
         <f t="shared" si="0"/>
         <v>97.3095</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A10" s="29" t="s">
+      <c r="H9" s="54">
+        <v>2022</v>
+      </c>
+      <c r="I9" s="49">
+        <v>1473.8717942959731</v>
+      </c>
+      <c r="J9" s="29">
+        <v>3380</v>
+      </c>
+      <c r="K9" s="50">
+        <f t="shared" ref="K9:K12" si="1">(I9-J9)/J9</f>
+        <v>-0.56394325612545171</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A10" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="18">
+      <c r="B10" s="15">
         <v>36.92</v>
       </c>
-      <c r="C10" s="19">
+      <c r="C10" s="16">
         <v>53.64</v>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="16">
         <v>53.64</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="16">
         <v>53.64</v>
       </c>
-      <c r="F10" s="20">
+      <c r="F10" s="17">
         <f t="shared" si="0"/>
         <v>49.459999999999994</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A11" s="29" t="s">
+      <c r="H10" s="54">
+        <v>2023</v>
+      </c>
+      <c r="I10" s="49">
+        <v>1685.4106346098099</v>
+      </c>
+      <c r="J10" s="29">
+        <v>3320</v>
+      </c>
+      <c r="K10" s="50">
+        <f t="shared" si="1"/>
+        <v>-0.49234619439463556</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="18">
+      <c r="B11" s="15">
         <v>58.08</v>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="16">
         <v>84.36</v>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="16">
         <v>84.36</v>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="16">
         <v>84.36</v>
       </c>
-      <c r="F11" s="20">
+      <c r="F11" s="17">
         <f t="shared" si="0"/>
         <v>77.790000000000006</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A12" s="29" t="s">
+      <c r="H11" s="55">
+        <v>2024</v>
+      </c>
+      <c r="I11" s="51">
+        <v>2156.7417637150811</v>
+      </c>
+      <c r="J11" s="38">
+        <v>3030</v>
+      </c>
+      <c r="K11" s="52">
+        <f t="shared" si="1"/>
+        <v>-0.28820403837786102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="18">
+      <c r="B12" s="15">
         <v>265.31358231668298</v>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="16">
         <v>298.12579429597298</v>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="16">
         <v>214.02563460981</v>
       </c>
-      <c r="E12" s="19">
+      <c r="E12" s="16">
         <v>583.71476371508106</v>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="17">
         <f t="shared" si="0"/>
         <v>340.29494373438672</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="14" t="s">
+      <c r="H12" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="I12" s="56">
+        <f>SUM(_xlfn.ANCHORARRAY(I8))</f>
+        <v>6855.820774937547</v>
+      </c>
+      <c r="J12" s="57">
+        <f>SUM(J8:J11)</f>
+        <v>12640</v>
+      </c>
+      <c r="K12" s="58">
+        <f t="shared" si="1"/>
+        <v>-0.45760911590683961</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B13" s="21">
+      <c r="B13" s="18">
         <v>249</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="19">
         <v>284</v>
       </c>
-      <c r="D13" s="22">
+      <c r="D13" s="19">
         <v>461</v>
       </c>
-      <c r="E13" s="22">
+      <c r="E13" s="19">
         <v>461</v>
       </c>
-      <c r="F13" s="23">
+      <c r="F13" s="20">
         <f t="shared" si="0"/>
         <v>363.75</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="14" t="s">
+    <row r="14" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="24">
+      <c r="B14" s="21">
         <f>SUM(B5:B13)</f>
         <v>1539.7965823166828</v>
       </c>
-      <c r="C14" s="25">
-        <f t="shared" ref="C14:E14" si="1">SUM(C5:C13)</f>
+      <c r="C14" s="22">
+        <f t="shared" ref="C14:E14" si="2">SUM(C5:C13)</f>
         <v>1473.8717942959731</v>
       </c>
-      <c r="D14" s="25">
-        <f t="shared" si="1"/>
+      <c r="D14" s="22">
+        <f t="shared" si="2"/>
         <v>1685.4106346098099</v>
       </c>
-      <c r="E14" s="26">
-        <f t="shared" si="1"/>
+      <c r="E14" s="23">
+        <f t="shared" si="2"/>
         <v>2156.7417637150811</v>
       </c>
-      <c r="F14" s="23">
-        <f t="shared" ref="F14" si="2">SUM(F5:F13)</f>
+      <c r="F14" s="20">
+        <f t="shared" ref="F14" si="3">SUM(F5:F13)</f>
         <v>1713.9551937343867</v>
       </c>
     </row>
@@ -1522,52 +1672,52 @@
       </c>
     </row>
     <row r="19" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="35"/>
-      <c r="B19" s="6" t="s">
+      <c r="A19" s="31"/>
+      <c r="B19" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="35"/>
+      <c r="C19" s="44"/>
+      <c r="D19" s="44"/>
+      <c r="E19" s="44"/>
+      <c r="F19" s="31"/>
     </row>
     <row r="20" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="39" t="s">
+      <c r="A20" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="8">
         <v>2021</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="8">
         <v>2022</v>
       </c>
-      <c r="D20" s="11">
+      <c r="D20" s="8">
         <v>2023</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="8">
         <v>2024</v>
       </c>
-      <c r="F20" s="40" t="s">
+      <c r="F20" s="36" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A21" s="36" t="s">
+      <c r="A21" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="16">
         <v>118.18600000000001</v>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="16">
         <v>74.753</v>
       </c>
-      <c r="D21" s="19">
+      <c r="D21" s="16">
         <v>128.80199999999999</v>
       </c>
-      <c r="E21" s="19">
+      <c r="E21" s="16">
         <v>82.938999999999993</v>
       </c>
-      <c r="F21" s="20">
+      <c r="F21" s="17">
         <f>AVERAGE(B21:E21)</f>
         <v>101.16999999999999</v>
       </c>
@@ -1577,149 +1727,149 @@
       <c r="Z21" s="2"/>
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A22" s="36" t="s">
+      <c r="A22" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="19">
+      <c r="B22" s="16">
         <v>100.309</v>
       </c>
-      <c r="C22" s="19">
+      <c r="C22" s="16">
         <v>98.667000000000002</v>
       </c>
-      <c r="D22" s="19">
+      <c r="D22" s="16">
         <v>80.421000000000006</v>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="16">
         <v>176.49799999999999</v>
       </c>
-      <c r="F22" s="20">
-        <f t="shared" ref="F22:F29" si="3">AVERAGE(B22:E22)</f>
+      <c r="F22" s="17">
+        <f t="shared" ref="F22:F29" si="4">AVERAGE(B22:E22)</f>
         <v>113.97375</v>
       </c>
     </row>
     <row r="23" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A23" s="36" t="s">
+      <c r="A23" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="19">
+      <c r="B23" s="16">
         <v>551.13499999999999</v>
       </c>
-      <c r="C23" s="19">
+      <c r="C23" s="16">
         <v>464.16500000000002</v>
       </c>
-      <c r="D23" s="19">
+      <c r="D23" s="16">
         <v>525.50099999999998</v>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="16">
         <v>577.67599999999993</v>
       </c>
-      <c r="F23" s="20">
-        <f t="shared" si="3"/>
+      <c r="F23" s="17">
+        <f t="shared" si="4"/>
         <v>529.61924999999997</v>
       </c>
     </row>
     <row r="24" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A24" s="36" t="s">
+      <c r="A24" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="B24" s="19">
+      <c r="B24" s="16">
         <v>71.613</v>
       </c>
-      <c r="C24" s="19">
+      <c r="C24" s="16">
         <v>36.423000000000002</v>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="16">
         <v>27.530999999999999</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="16">
         <v>26.783999999999999</v>
       </c>
-      <c r="F24" s="20">
-        <f t="shared" si="3"/>
+      <c r="F24" s="17">
+        <f t="shared" si="4"/>
         <v>40.58775</v>
       </c>
     </row>
     <row r="25" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A25" s="36" t="s">
+      <c r="A25" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="19">
+      <c r="B25" s="16">
         <v>89.24</v>
       </c>
-      <c r="C25" s="19">
+      <c r="C25" s="16">
         <v>79.738</v>
       </c>
-      <c r="D25" s="19">
+      <c r="D25" s="16">
         <v>110.13000000000001</v>
       </c>
-      <c r="E25" s="19">
+      <c r="E25" s="16">
         <v>110.13000000000001</v>
       </c>
-      <c r="F25" s="20">
-        <f t="shared" si="3"/>
+      <c r="F25" s="17">
+        <f t="shared" si="4"/>
         <v>97.3095</v>
       </c>
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A26" s="36" t="s">
+      <c r="A26" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B26" s="19">
+      <c r="B26" s="16">
         <v>36.92</v>
       </c>
-      <c r="C26" s="19">
+      <c r="C26" s="16">
         <v>53.64</v>
       </c>
-      <c r="D26" s="19">
+      <c r="D26" s="16">
         <v>53.64</v>
       </c>
-      <c r="E26" s="19">
+      <c r="E26" s="16">
         <v>53.64</v>
       </c>
-      <c r="F26" s="20">
-        <f t="shared" si="3"/>
+      <c r="F26" s="17">
+        <f t="shared" si="4"/>
         <v>49.459999999999994</v>
       </c>
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A27" s="36" t="s">
+      <c r="A27" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B27" s="19">
+      <c r="B27" s="16">
         <v>58.08</v>
       </c>
-      <c r="C27" s="19">
+      <c r="C27" s="16">
         <v>84.36</v>
       </c>
-      <c r="D27" s="19">
+      <c r="D27" s="16">
         <v>84.36</v>
       </c>
-      <c r="E27" s="19">
+      <c r="E27" s="16">
         <v>84.36</v>
       </c>
-      <c r="F27" s="20">
-        <f t="shared" si="3"/>
+      <c r="F27" s="17">
+        <f t="shared" si="4"/>
         <v>77.790000000000006</v>
       </c>
     </row>
     <row r="28" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A28" s="36" t="s">
+      <c r="A28" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B28" s="19">
+      <c r="B28" s="16">
         <v>256.49358231668299</v>
       </c>
-      <c r="C28" s="19">
+      <c r="C28" s="16">
         <v>288.540794295973</v>
       </c>
-      <c r="D28" s="19">
+      <c r="D28" s="16">
         <v>207.28263460981</v>
       </c>
-      <c r="E28" s="19">
+      <c r="E28" s="16">
         <v>565.12376371508105</v>
       </c>
-      <c r="F28" s="20">
-        <f t="shared" si="3"/>
+      <c r="F28" s="17">
+        <f t="shared" si="4"/>
         <v>329.36019373438671</v>
       </c>
       <c r="G28" t="s">
@@ -1727,48 +1877,48 @@
       </c>
     </row>
     <row r="29" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="37" t="s">
+      <c r="A29" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="B29" s="22">
+      <c r="B29" s="19">
         <v>249</v>
       </c>
-      <c r="C29" s="22">
+      <c r="C29" s="19">
         <v>284</v>
       </c>
-      <c r="D29" s="22">
+      <c r="D29" s="19">
         <v>461</v>
       </c>
-      <c r="E29" s="22">
+      <c r="E29" s="19">
         <v>461</v>
       </c>
-      <c r="F29" s="20">
-        <f t="shared" si="3"/>
+      <c r="F29" s="17">
+        <f t="shared" si="4"/>
         <v>363.75</v>
       </c>
     </row>
     <row r="30" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="37" t="s">
+      <c r="A30" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="22">
+      <c r="B30" s="19">
         <f>SUM(B21:B29)</f>
         <v>1530.9765823166829</v>
       </c>
-      <c r="C30" s="22">
-        <f t="shared" ref="C30:F30" si="4">SUM(C21:C29)</f>
+      <c r="C30" s="19">
+        <f t="shared" ref="C30:F30" si="5">SUM(C21:C29)</f>
         <v>1464.2867942959731</v>
       </c>
-      <c r="D30" s="22">
-        <f t="shared" si="4"/>
+      <c r="D30" s="19">
+        <f t="shared" si="5"/>
         <v>1678.66763460981</v>
       </c>
-      <c r="E30" s="22">
-        <f t="shared" si="4"/>
+      <c r="E30" s="19">
+        <f t="shared" si="5"/>
         <v>2138.1507637150808</v>
       </c>
-      <c r="F30" s="41">
-        <f t="shared" si="4"/>
+      <c r="F30" s="37">
+        <f t="shared" si="5"/>
         <v>1703.0204437343866</v>
       </c>
     </row>
@@ -1783,232 +1933,232 @@
       </c>
     </row>
     <row r="36" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="35"/>
-      <c r="B36" s="6" t="s">
+      <c r="A36" s="31"/>
+      <c r="B36" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="35"/>
+      <c r="C36" s="44"/>
+      <c r="D36" s="44"/>
+      <c r="E36" s="44"/>
+      <c r="F36" s="31"/>
     </row>
     <row r="37" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="39" t="s">
+      <c r="A37" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="8">
         <v>2021</v>
       </c>
-      <c r="C37" s="11">
+      <c r="C37" s="8">
         <v>2022</v>
       </c>
-      <c r="D37" s="11">
+      <c r="D37" s="8">
         <v>2023</v>
       </c>
-      <c r="E37" s="11">
+      <c r="E37" s="8">
         <v>2024</v>
       </c>
-      <c r="F37" s="40" t="s">
+      <c r="F37" s="36" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A38" s="36" t="s">
+      <c r="A38" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B38" s="19">
+      <c r="B38" s="16">
         <f>B67</f>
         <v>118.18600000000001</v>
       </c>
-      <c r="C38" s="19">
-        <f t="shared" ref="C38:E38" si="5">C67</f>
+      <c r="C38" s="16">
+        <f t="shared" ref="C38:E38" si="6">C67</f>
         <v>74.753</v>
       </c>
-      <c r="D38" s="19">
-        <f t="shared" si="5"/>
+      <c r="D38" s="16">
+        <f t="shared" si="6"/>
         <v>128.80199999999999</v>
       </c>
-      <c r="E38" s="19">
-        <f t="shared" si="5"/>
+      <c r="E38" s="16">
+        <f t="shared" si="6"/>
         <v>82.938999999999993</v>
       </c>
-      <c r="F38" s="20">
+      <c r="F38" s="17">
         <f>AVERAGE(B38:E38)</f>
         <v>101.16999999999999</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A39" s="36" t="s">
+      <c r="A39" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B39" s="19">
+      <c r="B39" s="16">
         <f>B68</f>
         <v>100.309</v>
       </c>
-      <c r="C39" s="19">
-        <f t="shared" ref="C39:E39" si="6">C68</f>
+      <c r="C39" s="16">
+        <f t="shared" ref="C39:E39" si="7">C68</f>
         <v>98.667000000000002</v>
       </c>
-      <c r="D39" s="19">
-        <f t="shared" si="6"/>
+      <c r="D39" s="16">
+        <f t="shared" si="7"/>
         <v>80.421000000000006</v>
       </c>
-      <c r="E39" s="19">
-        <f t="shared" si="6"/>
+      <c r="E39" s="16">
+        <f t="shared" si="7"/>
         <v>176.49799999999999</v>
       </c>
-      <c r="F39" s="20">
-        <f t="shared" ref="F39:F46" si="7">AVERAGE(B39:E39)</f>
+      <c r="F39" s="17">
+        <f t="shared" ref="F39:F46" si="8">AVERAGE(B39:E39)</f>
         <v>113.97375</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A40" s="36" t="s">
+      <c r="A40" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B40" s="19">
+      <c r="B40" s="16">
         <f>B56+B69</f>
         <v>551.13499999999999</v>
       </c>
-      <c r="C40" s="19">
-        <f t="shared" ref="C40:E40" si="8">C56+C69</f>
+      <c r="C40" s="16">
+        <f t="shared" ref="C40:E40" si="9">C56+C69</f>
         <v>464.16500000000002</v>
       </c>
-      <c r="D40" s="19">
+      <c r="D40" s="16">
+        <f t="shared" si="9"/>
+        <v>525.50099999999998</v>
+      </c>
+      <c r="E40" s="16">
+        <f t="shared" si="9"/>
+        <v>577.67599999999993</v>
+      </c>
+      <c r="F40" s="17">
         <f t="shared" si="8"/>
-        <v>525.50099999999998</v>
-      </c>
-      <c r="E40" s="19">
-        <f t="shared" si="8"/>
-        <v>577.67599999999993</v>
-      </c>
-      <c r="F40" s="20">
-        <f t="shared" si="7"/>
         <v>529.61924999999997</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A41" s="36" t="s">
+      <c r="A41" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="B41" s="19">
+      <c r="B41" s="16">
         <f>B70</f>
         <v>71.613</v>
       </c>
-      <c r="C41" s="19">
-        <f t="shared" ref="C41:E41" si="9">C70</f>
+      <c r="C41" s="16">
+        <f t="shared" ref="C41:E41" si="10">C70</f>
         <v>36.423000000000002</v>
       </c>
-      <c r="D41" s="19">
-        <f t="shared" si="9"/>
+      <c r="D41" s="16">
+        <f t="shared" si="10"/>
         <v>27.530999999999999</v>
       </c>
-      <c r="E41" s="19">
-        <f t="shared" si="9"/>
+      <c r="E41" s="16">
+        <f t="shared" si="10"/>
         <v>26.783999999999999</v>
       </c>
-      <c r="F41" s="20">
-        <f t="shared" si="7"/>
+      <c r="F41" s="17">
+        <f t="shared" si="8"/>
         <v>40.58775</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A42" s="36" t="s">
+      <c r="A42" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="B42" s="19">
+      <c r="B42" s="16">
         <f>B71</f>
         <v>89.24</v>
       </c>
-      <c r="C42" s="19">
-        <f t="shared" ref="C42:E42" si="10">C71</f>
+      <c r="C42" s="16">
+        <f t="shared" ref="C42:E42" si="11">C71</f>
         <v>79.738</v>
       </c>
-      <c r="D42" s="19">
-        <f t="shared" si="10"/>
+      <c r="D42" s="16">
+        <f t="shared" si="11"/>
         <v>110.13000000000001</v>
       </c>
-      <c r="E42" s="19">
-        <f t="shared" si="10"/>
+      <c r="E42" s="16">
+        <f t="shared" si="11"/>
         <v>110.13000000000001</v>
       </c>
-      <c r="F42" s="20">
-        <f t="shared" si="7"/>
+      <c r="F42" s="17">
+        <f t="shared" si="8"/>
         <v>97.3095</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A43" s="36" t="s">
+      <c r="A43" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B43" s="19">
+      <c r="B43" s="16">
         <f>B72</f>
         <v>36.92</v>
       </c>
-      <c r="C43" s="19">
-        <f t="shared" ref="C43:E43" si="11">C72</f>
+      <c r="C43" s="16">
+        <f t="shared" ref="C43:E43" si="12">C72</f>
         <v>53.64</v>
       </c>
-      <c r="D43" s="19">
-        <f t="shared" si="11"/>
+      <c r="D43" s="16">
+        <f t="shared" si="12"/>
         <v>53.64</v>
       </c>
-      <c r="E43" s="19">
-        <f t="shared" si="11"/>
+      <c r="E43" s="16">
+        <f t="shared" si="12"/>
         <v>53.64</v>
       </c>
-      <c r="F43" s="20">
-        <f t="shared" si="7"/>
+      <c r="F43" s="17">
+        <f t="shared" si="8"/>
         <v>49.459999999999994</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A44" s="36" t="s">
+      <c r="A44" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B44" s="19">
+      <c r="B44" s="16">
         <f>B73</f>
         <v>58.08</v>
       </c>
-      <c r="C44" s="19">
-        <f t="shared" ref="C44:E44" si="12">C73</f>
+      <c r="C44" s="16">
+        <f t="shared" ref="C44:E44" si="13">C73</f>
         <v>84.36</v>
       </c>
-      <c r="D44" s="19">
-        <f t="shared" si="12"/>
+      <c r="D44" s="16">
+        <f t="shared" si="13"/>
         <v>84.36</v>
       </c>
-      <c r="E44" s="19">
-        <f t="shared" si="12"/>
+      <c r="E44" s="16">
+        <f t="shared" si="13"/>
         <v>84.36</v>
       </c>
-      <c r="F44" s="20">
-        <f t="shared" si="7"/>
+      <c r="F44" s="17">
+        <f t="shared" si="8"/>
         <v>77.790000000000006</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A45" s="36" t="s">
+      <c r="A45" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B45" s="19">
+      <c r="B45" s="16">
         <f>B57</f>
         <v>207</v>
       </c>
-      <c r="C45" s="19">
-        <f t="shared" ref="C45:E45" si="13">C57</f>
+      <c r="C45" s="16">
+        <f t="shared" ref="C45:E45" si="14">C57</f>
         <v>239</v>
       </c>
-      <c r="D45" s="19">
-        <f t="shared" si="13"/>
+      <c r="D45" s="16">
+        <f t="shared" si="14"/>
         <v>175</v>
       </c>
-      <c r="E45" s="19">
-        <f t="shared" si="13"/>
+      <c r="E45" s="16">
+        <f t="shared" si="14"/>
         <v>175</v>
       </c>
-      <c r="F45" s="20">
-        <f t="shared" si="7"/>
+      <c r="F45" s="17">
+        <f t="shared" si="8"/>
         <v>199</v>
       </c>
       <c r="G45" t="s">
@@ -2016,52 +2166,52 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A46" s="36" t="s">
+      <c r="A46" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B46" s="19">
+      <c r="B46" s="16">
         <f>B58</f>
         <v>249</v>
       </c>
-      <c r="C46" s="19">
-        <f t="shared" ref="C46:E46" si="14">C58</f>
+      <c r="C46" s="16">
+        <f t="shared" ref="C46:E46" si="15">C58</f>
         <v>284</v>
       </c>
-      <c r="D46" s="19">
-        <f t="shared" si="14"/>
+      <c r="D46" s="16">
+        <f t="shared" si="15"/>
         <v>461</v>
       </c>
-      <c r="E46" s="19">
-        <f t="shared" si="14"/>
+      <c r="E46" s="16">
+        <f t="shared" si="15"/>
         <v>461</v>
       </c>
-      <c r="F46" s="20">
-        <f t="shared" si="7"/>
+      <c r="F46" s="17">
+        <f t="shared" si="8"/>
         <v>363.75</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="40" t="s">
+      <c r="A47" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="25">
+      <c r="B47" s="22">
         <f>SUM(B38:B46)</f>
         <v>1481.4829999999999</v>
       </c>
-      <c r="C47" s="25">
-        <f t="shared" ref="C47:F47" si="15">SUM(C38:C46)</f>
+      <c r="C47" s="22">
+        <f t="shared" ref="C47:F47" si="16">SUM(C38:C46)</f>
         <v>1414.7460000000001</v>
       </c>
-      <c r="D47" s="25">
-        <f t="shared" si="15"/>
+      <c r="D47" s="22">
+        <f t="shared" si="16"/>
         <v>1646.3849999999998</v>
       </c>
-      <c r="E47" s="25">
-        <f t="shared" si="15"/>
+      <c r="E47" s="22">
+        <f t="shared" si="16"/>
         <v>1748.0269999999998</v>
       </c>
-      <c r="F47" s="41">
-        <f t="shared" si="15"/>
+      <c r="F47" s="37">
+        <f t="shared" si="16"/>
         <v>1572.6602499999999</v>
       </c>
     </row>
@@ -2074,171 +2224,171 @@
       </c>
     </row>
     <row r="53" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A53" s="48" t="s">
+      <c r="A53" s="42" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A54" s="28"/>
-      <c r="B54" s="43" t="s">
+      <c r="A54" s="25"/>
+      <c r="B54" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C54" s="32"/>
-      <c r="D54" s="32"/>
-      <c r="E54" s="44"/>
-      <c r="F54" s="13"/>
+      <c r="C54" s="47"/>
+      <c r="D54" s="47"/>
+      <c r="E54" s="48"/>
+      <c r="F54" s="10"/>
     </row>
     <row r="55" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A55" s="47" t="s">
+      <c r="A55" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="B55" s="10">
+      <c r="B55" s="7">
         <v>2021</v>
       </c>
-      <c r="C55" s="11">
+      <c r="C55" s="8">
         <v>2022</v>
       </c>
-      <c r="D55" s="11">
+      <c r="D55" s="8">
         <v>2023</v>
       </c>
-      <c r="E55" s="12">
+      <c r="E55" s="9">
         <v>2024</v>
       </c>
-      <c r="F55" s="12" t="s">
+      <c r="F55" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A56" s="28" t="s">
+      <c r="A56" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B56" s="28">
+      <c r="B56" s="25">
         <v>139</v>
       </c>
-      <c r="C56" s="30">
+      <c r="C56" s="27">
         <v>100</v>
       </c>
-      <c r="D56" s="30">
+      <c r="D56" s="27">
         <v>89</v>
       </c>
-      <c r="E56" s="13">
+      <c r="E56" s="10">
         <v>89</v>
       </c>
-      <c r="F56" s="46">
+      <c r="F56" s="40">
         <f>AVERAGE(B56:E56)</f>
         <v>104.25</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A57" s="29" t="s">
+      <c r="A57" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B57" s="29">
+      <c r="B57" s="26">
         <v>207</v>
       </c>
-      <c r="C57" s="33">
+      <c r="C57" s="29">
         <v>239</v>
       </c>
-      <c r="D57" s="33">
+      <c r="D57" s="29">
         <v>175</v>
       </c>
-      <c r="E57" s="34">
+      <c r="E57" s="30">
         <v>175</v>
       </c>
-      <c r="F57" s="31">
-        <f t="shared" ref="F57:F61" si="16">AVERAGE(B57:E57)</f>
+      <c r="F57" s="28">
+        <f t="shared" ref="F57:F61" si="17">AVERAGE(B57:E57)</f>
         <v>199</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A58" s="29" t="s">
+      <c r="A58" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="B58" s="29">
+      <c r="B58" s="26">
         <v>249</v>
       </c>
-      <c r="C58" s="33">
+      <c r="C58" s="29">
         <v>284</v>
       </c>
-      <c r="D58" s="33">
+      <c r="D58" s="29">
         <v>461</v>
       </c>
-      <c r="E58" s="34">
+      <c r="E58" s="30">
         <v>461</v>
       </c>
-      <c r="F58" s="31">
-        <f t="shared" si="16"/>
+      <c r="F58" s="28">
+        <f t="shared" si="17"/>
         <v>363.75</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A59" s="29" t="s">
+      <c r="A59" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B59" s="29">
+      <c r="B59" s="26">
         <f>SUM(B56:B58)</f>
         <v>595</v>
       </c>
-      <c r="C59" s="33">
-        <f t="shared" ref="C59:E59" si="17">SUM(C56:C58)</f>
+      <c r="C59" s="29">
+        <f t="shared" ref="C59:E59" si="18">SUM(C56:C58)</f>
         <v>623</v>
       </c>
-      <c r="D59" s="33">
+      <c r="D59" s="29">
+        <f t="shared" si="18"/>
+        <v>725</v>
+      </c>
+      <c r="E59" s="30">
+        <f t="shared" si="18"/>
+        <v>725</v>
+      </c>
+      <c r="F59" s="28">
         <f t="shared" si="17"/>
-        <v>725</v>
-      </c>
-      <c r="E59" s="34">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A60" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B60" s="11">
+        <v>1091</v>
+      </c>
+      <c r="C60" s="38">
+        <v>804</v>
+      </c>
+      <c r="D60" s="38">
+        <v>836</v>
+      </c>
+      <c r="E60" s="39">
+        <v>836</v>
+      </c>
+      <c r="F60" s="24">
         <f t="shared" si="17"/>
-        <v>725</v>
-      </c>
-      <c r="F59" s="31">
-        <f t="shared" si="16"/>
-        <v>667</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A60" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="B60" s="14">
-        <v>1091</v>
-      </c>
-      <c r="C60" s="42">
-        <v>804</v>
-      </c>
-      <c r="D60" s="42">
-        <v>836</v>
-      </c>
-      <c r="E60" s="45">
-        <v>836</v>
-      </c>
-      <c r="F60" s="27">
-        <f t="shared" si="16"/>
         <v>891.75</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A61" s="14" t="s">
+      <c r="A61" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B61" s="14">
+      <c r="B61" s="11">
         <f>SUM(B59:B60)</f>
         <v>1686</v>
       </c>
-      <c r="C61" s="42">
-        <f t="shared" ref="C61:E61" si="18">SUM(C59:C60)</f>
+      <c r="C61" s="38">
+        <f t="shared" ref="C61:E61" si="19">SUM(C59:C60)</f>
         <v>1427</v>
       </c>
-      <c r="D61" s="42">
-        <f t="shared" si="18"/>
+      <c r="D61" s="38">
+        <f t="shared" si="19"/>
         <v>1561</v>
       </c>
-      <c r="E61" s="45">
-        <f t="shared" si="18"/>
+      <c r="E61" s="39">
+        <f t="shared" si="19"/>
         <v>1561</v>
       </c>
-      <c r="F61" s="27">
-        <f t="shared" si="16"/>
+      <c r="F61" s="24">
+        <f t="shared" si="17"/>
         <v>1558.75</v>
       </c>
     </row>
@@ -2248,209 +2398,209 @@
       </c>
     </row>
     <row r="64" spans="1:6" ht="13.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A64" s="48" t="s">
+      <c r="A64" s="42" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A65" s="38"/>
-      <c r="B65" s="32" t="s">
+      <c r="A65" s="34"/>
+      <c r="B65" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="C65" s="32"/>
-      <c r="D65" s="32"/>
-      <c r="E65" s="32"/>
-      <c r="F65" s="38"/>
+      <c r="C65" s="47"/>
+      <c r="D65" s="47"/>
+      <c r="E65" s="47"/>
+      <c r="F65" s="34"/>
     </row>
     <row r="66" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A66" s="39" t="s">
+      <c r="A66" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B66" s="11">
+      <c r="B66" s="8">
         <v>2021</v>
       </c>
-      <c r="C66" s="11">
+      <c r="C66" s="8">
         <v>2022</v>
       </c>
-      <c r="D66" s="11">
+      <c r="D66" s="8">
         <v>2023</v>
       </c>
-      <c r="E66" s="11">
+      <c r="E66" s="8">
         <v>2024</v>
       </c>
-      <c r="F66" s="40" t="s">
+      <c r="F66" s="36" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A67" s="36" t="s">
+      <c r="A67" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B67" s="19">
+      <c r="B67" s="16">
         <v>118.18600000000001</v>
       </c>
-      <c r="C67" s="19">
+      <c r="C67" s="16">
         <v>74.753</v>
       </c>
-      <c r="D67" s="19">
+      <c r="D67" s="16">
         <v>128.80199999999999</v>
       </c>
-      <c r="E67" s="19">
+      <c r="E67" s="16">
         <v>82.938999999999993</v>
       </c>
-      <c r="F67" s="20">
+      <c r="F67" s="17">
         <f>AVERAGE(B67:E67)</f>
         <v>101.16999999999999</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A68" s="36" t="s">
+      <c r="A68" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B68" s="19">
+      <c r="B68" s="16">
         <v>100.309</v>
       </c>
-      <c r="C68" s="19">
+      <c r="C68" s="16">
         <v>98.667000000000002</v>
       </c>
-      <c r="D68" s="19">
+      <c r="D68" s="16">
         <v>80.421000000000006</v>
       </c>
-      <c r="E68" s="19">
+      <c r="E68" s="16">
         <v>176.49799999999999</v>
       </c>
-      <c r="F68" s="20">
-        <f t="shared" ref="F68:F74" si="19">AVERAGE(B68:E68)</f>
+      <c r="F68" s="17">
+        <f t="shared" ref="F68:F74" si="20">AVERAGE(B68:E68)</f>
         <v>113.97375</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A69" s="36" t="s">
+      <c r="A69" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B69" s="19">
+      <c r="B69" s="16">
         <v>412.13499999999999</v>
       </c>
-      <c r="C69" s="19">
+      <c r="C69" s="16">
         <v>364.16500000000002</v>
       </c>
-      <c r="D69" s="19">
+      <c r="D69" s="16">
         <v>436.50100000000003</v>
       </c>
-      <c r="E69" s="19">
+      <c r="E69" s="16">
         <v>488.67599999999999</v>
       </c>
-      <c r="F69" s="20">
-        <f t="shared" si="19"/>
+      <c r="F69" s="17">
+        <f t="shared" si="20"/>
         <v>425.36924999999997</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A70" s="36" t="s">
+      <c r="A70" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="B70" s="19">
+      <c r="B70" s="16">
         <v>71.613</v>
       </c>
-      <c r="C70" s="19">
+      <c r="C70" s="16">
         <v>36.423000000000002</v>
       </c>
-      <c r="D70" s="19">
+      <c r="D70" s="16">
         <v>27.530999999999999</v>
       </c>
-      <c r="E70" s="19">
+      <c r="E70" s="16">
         <v>26.783999999999999</v>
       </c>
-      <c r="F70" s="20">
-        <f t="shared" si="19"/>
+      <c r="F70" s="17">
+        <f t="shared" si="20"/>
         <v>40.58775</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A71" s="36" t="s">
+      <c r="A71" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="B71" s="19">
+      <c r="B71" s="16">
         <v>89.24</v>
       </c>
-      <c r="C71" s="19">
+      <c r="C71" s="16">
         <v>79.738</v>
       </c>
-      <c r="D71" s="19">
+      <c r="D71" s="16">
         <v>110.13000000000001</v>
       </c>
-      <c r="E71" s="19">
+      <c r="E71" s="16">
         <v>110.13000000000001</v>
       </c>
-      <c r="F71" s="20">
-        <f t="shared" si="19"/>
+      <c r="F71" s="17">
+        <f t="shared" si="20"/>
         <v>97.3095</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A72" s="36" t="s">
+      <c r="A72" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B72" s="19">
+      <c r="B72" s="16">
         <v>36.92</v>
       </c>
-      <c r="C72" s="19">
+      <c r="C72" s="16">
         <v>53.64</v>
       </c>
-      <c r="D72" s="19">
+      <c r="D72" s="16">
         <v>53.64</v>
       </c>
-      <c r="E72" s="19">
+      <c r="E72" s="16">
         <v>53.64</v>
       </c>
-      <c r="F72" s="20">
-        <f t="shared" si="19"/>
+      <c r="F72" s="17">
+        <f t="shared" si="20"/>
         <v>49.459999999999994</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A73" s="37" t="s">
+      <c r="A73" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="B73" s="22">
+      <c r="B73" s="19">
         <v>58.08</v>
       </c>
-      <c r="C73" s="22">
+      <c r="C73" s="19">
         <v>84.36</v>
       </c>
-      <c r="D73" s="22">
+      <c r="D73" s="19">
         <v>84.36</v>
       </c>
-      <c r="E73" s="22">
+      <c r="E73" s="19">
         <v>84.36</v>
       </c>
-      <c r="F73" s="23">
-        <f t="shared" si="19"/>
+      <c r="F73" s="20">
+        <f t="shared" si="20"/>
         <v>77.790000000000006</v>
       </c>
     </row>
     <row r="74" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A74" s="37" t="s">
+      <c r="A74" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="B74" s="22">
+      <c r="B74" s="19">
         <f>SUM(B67:B73)</f>
         <v>886.48299999999995</v>
       </c>
-      <c r="C74" s="22">
-        <f t="shared" ref="C74:E74" si="20">SUM(C67:C73)</f>
+      <c r="C74" s="19">
+        <f t="shared" ref="C74:E74" si="21">SUM(C67:C73)</f>
         <v>791.74600000000009</v>
       </c>
-      <c r="D74" s="22">
+      <c r="D74" s="19">
+        <f t="shared" si="21"/>
+        <v>921.38499999999999</v>
+      </c>
+      <c r="E74" s="19">
+        <f t="shared" si="21"/>
+        <v>1023.027</v>
+      </c>
+      <c r="F74" s="20">
         <f t="shared" si="20"/>
-        <v>921.38499999999999</v>
-      </c>
-      <c r="E74" s="22">
-        <f t="shared" si="20"/>
-        <v>1023.027</v>
-      </c>
-      <c r="F74" s="23">
-        <f t="shared" si="19"/>
         <v>905.66025000000002</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2025 MLS projection documents
</commit_message>
<xml_diff>
--- a/2025-MLS-projections/BSIA Catch/2021-2024 BSIA MLS Catch.xlsx
+++ b/2025-MLS-projections/BSIA Catch/2021-2024 BSIA MLS Catch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jon.brodziak\Desktop\2024 WCNPO MLS Rebuilding\2025 MLS projections\BSIA Catch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81961F3B-ACFB-4A6E-93B6-689BB6A2BD4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{393BBA42-5C37-437D-856C-9BAAF57CBFEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="16663" windowHeight="8863" firstSheet="1" activeTab="3" xr2:uid="{416E3EAD-1861-4C87-937B-DDBEC44D9B39}"/>
+    <workbookView xWindow="720" yWindow="326" windowWidth="13766" windowHeight="8185" firstSheet="2" activeTab="3" xr2:uid="{416E3EAD-1861-4C87-937B-DDBEC44D9B39}"/>
   </bookViews>
   <sheets>
     <sheet name="2021-2024-mls-catch" sheetId="4" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="37">
   <si>
     <t>G3</t>
   </si>
@@ -139,13 +139,37 @@
     <t>Total BSIA for WCNPO MLS Catch Biomass by Fleet Group</t>
   </si>
   <si>
-    <t>Observed</t>
-  </si>
-  <si>
     <t>F-Based</t>
   </si>
   <si>
     <t>% Change</t>
+  </si>
+  <si>
+    <t>F-Based Std</t>
+  </si>
+  <si>
+    <t>Observed C</t>
+  </si>
+  <si>
+    <t>Observed F</t>
+  </si>
+  <si>
+    <t>Obs F Std</t>
+  </si>
+  <si>
+    <t>F-Based C</t>
+  </si>
+  <si>
+    <t>Scenario 6</t>
+  </si>
+  <si>
+    <t>Scenario 1</t>
+  </si>
+  <si>
+    <t>F-Based 80CI</t>
+  </si>
+  <si>
+    <t>Obs F 80CI</t>
   </si>
 </sst>
 </file>
@@ -375,7 +399,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -491,6 +515,42 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -509,34 +569,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1304,7 +1349,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAC168C6-DF10-449B-94B3-ED91F02DF6B4}">
-  <dimension ref="A1:Z74"/>
+  <dimension ref="A1:AA74"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="18.07421875" customWidth="1"/>
@@ -1313,41 +1358,60 @@
     <col min="6" max="6" width="12.765625" customWidth="1"/>
     <col min="7" max="7" width="4.69140625" customWidth="1"/>
     <col min="8" max="8" width="7" customWidth="1"/>
-    <col min="9" max="9" width="9.53515625" customWidth="1"/>
+    <col min="9" max="9" width="10.69140625" customWidth="1"/>
     <col min="10" max="10" width="9.4609375" customWidth="1"/>
-    <col min="11" max="11" width="10.61328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.84375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="2.69140625" customWidth="1"/>
-    <col min="14" max="14" width="6.84375" customWidth="1"/>
-    <col min="16" max="16" width="6.07421875" customWidth="1"/>
-    <col min="17" max="17" width="10.4609375" customWidth="1"/>
-    <col min="19" max="19" width="3.3828125" customWidth="1"/>
-    <col min="20" max="20" width="7.61328125" customWidth="1"/>
-    <col min="25" max="25" width="4.3828125" customWidth="1"/>
-    <col min="26" max="26" width="7.53515625" customWidth="1"/>
+    <col min="11" max="11" width="11.3046875" customWidth="1"/>
+    <col min="12" max="12" width="10.61328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.84375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.07421875" customWidth="1"/>
+    <col min="15" max="15" width="6.84375" customWidth="1"/>
+    <col min="17" max="17" width="6.07421875" customWidth="1"/>
+    <col min="18" max="18" width="10.4609375" customWidth="1"/>
+    <col min="20" max="20" width="3.3828125" customWidth="1"/>
+    <col min="21" max="21" width="7.61328125" customWidth="1"/>
+    <col min="26" max="26" width="4.3828125" customWidth="1"/>
+    <col min="27" max="27" width="7.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="20.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:14" ht="20.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4"/>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="45"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="57"/>
       <c r="F3" s="5"/>
-    </row>
-    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="H3" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3" s="49" t="s">
+        <v>27</v>
+      </c>
+      <c r="N3" s="36" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="6" t="s">
         <v>4</v>
       </c>
@@ -1366,8 +1430,29 @@
       <c r="F4" s="10" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="H4" s="50">
+        <v>2021</v>
+      </c>
+      <c r="I4" s="45" cm="1">
+        <f t="array" ref="I4:I7">TRANSPOSE(B14:E14)</f>
+        <v>1539.7965823166828</v>
+      </c>
+      <c r="J4" s="29">
+        <v>2970</v>
+      </c>
+      <c r="K4" s="45">
+        <f>N4*1.28</f>
+        <v>614.4</v>
+      </c>
+      <c r="L4" s="46">
+        <f>(I4-J4)/J4</f>
+        <v>-0.48154997228394519</v>
+      </c>
+      <c r="N4" s="32">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5" s="25" t="s">
         <v>5</v>
       </c>
@@ -1387,8 +1472,28 @@
         <f>AVERAGE(B5:E5)</f>
         <v>101.16999999999999</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="H5" s="50">
+        <v>2022</v>
+      </c>
+      <c r="I5" s="45">
+        <v>1473.8717942959731</v>
+      </c>
+      <c r="J5" s="29">
+        <v>3420</v>
+      </c>
+      <c r="K5" s="45">
+        <f t="shared" ref="K5:K7" si="0">N5*1.28</f>
+        <v>729.6</v>
+      </c>
+      <c r="L5" s="46">
+        <f t="shared" ref="L5:L8" si="1">(I5-J5)/J5</f>
+        <v>-0.56904333500117743</v>
+      </c>
+      <c r="N5" s="32">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6" s="26" t="s">
         <v>6</v>
       </c>
@@ -1405,11 +1510,31 @@
         <v>176.49799999999999</v>
       </c>
       <c r="F6" s="17">
-        <f t="shared" ref="F6:F13" si="0">AVERAGE(B6:E6)</f>
+        <f t="shared" ref="F6:F13" si="2">AVERAGE(B6:E6)</f>
         <v>113.97375</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="H6" s="50">
+        <v>2023</v>
+      </c>
+      <c r="I6" s="45">
+        <v>1685.4106346098099</v>
+      </c>
+      <c r="J6" s="29">
+        <v>3380</v>
+      </c>
+      <c r="K6" s="45">
+        <f t="shared" si="0"/>
+        <v>857.6</v>
+      </c>
+      <c r="L6" s="46">
+        <f t="shared" si="1"/>
+        <v>-0.50135780041129885</v>
+      </c>
+      <c r="N6" s="32">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A7" s="26" t="s">
         <v>0</v>
       </c>
@@ -1426,23 +1551,31 @@
         <v>577.67599999999993</v>
       </c>
       <c r="F7" s="17">
+        <f t="shared" si="2"/>
+        <v>529.61924999999997</v>
+      </c>
+      <c r="H7" s="51">
+        <v>2024</v>
+      </c>
+      <c r="I7" s="47">
+        <v>2156.7417637150811</v>
+      </c>
+      <c r="J7" s="38">
+        <v>3080</v>
+      </c>
+      <c r="K7" s="45">
         <f t="shared" si="0"/>
-        <v>529.61924999999997</v>
-      </c>
-      <c r="H7" s="36" t="s">
-        <v>3</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" s="53" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
+        <v>896</v>
+      </c>
+      <c r="L7" s="48">
+        <f t="shared" si="1"/>
+        <v>-0.29975916762497368</v>
+      </c>
+      <c r="N7" s="33">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="26" t="s">
         <v>7</v>
       </c>
@@ -1459,25 +1592,29 @@
         <v>26.783999999999999</v>
       </c>
       <c r="F8" s="17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>40.58775</v>
       </c>
-      <c r="H8" s="54">
-        <v>2021</v>
-      </c>
-      <c r="I8" s="49" cm="1">
-        <f t="array" ref="I8:I11">TRANSPOSE(B14:E14)</f>
-        <v>1539.7965823166828</v>
-      </c>
-      <c r="J8" s="29">
-        <v>2910</v>
-      </c>
-      <c r="K8" s="50">
-        <f>(I8-J8)/J8</f>
-        <v>-0.47086028099083066</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="H8" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="I8" s="52">
+        <f>SUM(_xlfn.ANCHORARRAY(I4))</f>
+        <v>6855.820774937547</v>
+      </c>
+      <c r="J8" s="53">
+        <f>SUM(J4:J7)</f>
+        <v>12850</v>
+      </c>
+      <c r="K8" s="53" t="s">
+        <v>33</v>
+      </c>
+      <c r="L8" s="54">
+        <f t="shared" si="1"/>
+        <v>-0.46647309144454885</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A9" s="26" t="s">
         <v>8</v>
       </c>
@@ -1494,24 +1631,11 @@
         <v>110.13000000000001</v>
       </c>
       <c r="F9" s="17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>97.3095</v>
       </c>
-      <c r="H9" s="54">
-        <v>2022</v>
-      </c>
-      <c r="I9" s="49">
-        <v>1473.8717942959731</v>
-      </c>
-      <c r="J9" s="29">
-        <v>3380</v>
-      </c>
-      <c r="K9" s="50">
-        <f t="shared" ref="K9:K12" si="1">(I9-J9)/J9</f>
-        <v>-0.56394325612545171</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="10" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A10" s="26" t="s">
         <v>9</v>
       </c>
@@ -1528,24 +1652,29 @@
         <v>53.64</v>
       </c>
       <c r="F10" s="17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>49.459999999999994</v>
       </c>
-      <c r="H10" s="54">
-        <v>2023</v>
-      </c>
-      <c r="I10" s="49">
-        <v>1685.4106346098099</v>
-      </c>
-      <c r="J10" s="29">
-        <v>3320</v>
-      </c>
-      <c r="K10" s="50">
-        <f t="shared" si="1"/>
-        <v>-0.49234619439463556</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="H10" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="I10" s="43" t="s">
+        <v>30</v>
+      </c>
+      <c r="J10" s="43" t="s">
+        <v>36</v>
+      </c>
+      <c r="K10" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="L10" s="49" t="s">
+        <v>27</v>
+      </c>
+      <c r="N10" s="36" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11" s="26" t="s">
         <v>10</v>
       </c>
@@ -1562,24 +1691,31 @@
         <v>84.36</v>
       </c>
       <c r="F11" s="17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>77.790000000000006</v>
       </c>
-      <c r="H11" s="55">
-        <v>2024</v>
-      </c>
-      <c r="I11" s="51">
-        <v>2156.7417637150811</v>
-      </c>
-      <c r="J11" s="38">
-        <v>3030</v>
-      </c>
-      <c r="K11" s="52">
-        <f t="shared" si="1"/>
-        <v>-0.28820403837786102</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="H11" s="63">
+        <v>2021</v>
+      </c>
+      <c r="I11" s="64">
+        <v>0.52700000000000002</v>
+      </c>
+      <c r="J11" s="64">
+        <f>1.28*N11</f>
+        <v>0.1216</v>
+      </c>
+      <c r="K11" s="44">
+        <v>0.68</v>
+      </c>
+      <c r="L11" s="65">
+        <f>(I11-K11)/K11</f>
+        <v>-0.22500000000000003</v>
+      </c>
+      <c r="N11" s="32">
+        <v>9.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12" s="26" t="s">
         <v>1</v>
       </c>
@@ -1596,26 +1732,31 @@
         <v>583.71476371508106</v>
       </c>
       <c r="F12" s="17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>340.29494373438672</v>
       </c>
-      <c r="H12" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="I12" s="56">
-        <f>SUM(_xlfn.ANCHORARRAY(I8))</f>
-        <v>6855.820774937547</v>
-      </c>
-      <c r="J12" s="57">
-        <f>SUM(J8:J11)</f>
-        <v>12640</v>
-      </c>
-      <c r="K12" s="58">
-        <f t="shared" si="1"/>
-        <v>-0.45760911590683961</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="H12" s="50">
+        <v>2022</v>
+      </c>
+      <c r="I12" s="61">
+        <v>0.373</v>
+      </c>
+      <c r="J12" s="61">
+        <f t="shared" ref="J12:J14" si="3">1.28*N12</f>
+        <v>9.6000000000000002E-2</v>
+      </c>
+      <c r="K12" s="29">
+        <v>0.68</v>
+      </c>
+      <c r="L12" s="46">
+        <f t="shared" ref="L12:L14" si="4">(I12-K12)/K12</f>
+        <v>-0.45147058823529418</v>
+      </c>
+      <c r="N12" s="32">
+        <v>7.4999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A13" s="11" t="s">
         <v>2</v>
       </c>
@@ -1632,11 +1773,31 @@
         <v>461</v>
       </c>
       <c r="F13" s="20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>363.75</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="H13" s="50">
+        <v>2023</v>
+      </c>
+      <c r="I13" s="61">
+        <v>0.38100000000000001</v>
+      </c>
+      <c r="J13" s="61">
+        <f t="shared" si="3"/>
+        <v>0.11648</v>
+      </c>
+      <c r="K13" s="29">
+        <v>0.68</v>
+      </c>
+      <c r="L13" s="46">
+        <f t="shared" si="4"/>
+        <v>-0.43970588235294122</v>
+      </c>
+      <c r="N13" s="32">
+        <v>9.0999999999999998E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A14" s="11" t="s">
         <v>19</v>
       </c>
@@ -1645,43 +1806,68 @@
         <v>1539.7965823166828</v>
       </c>
       <c r="C14" s="22">
-        <f t="shared" ref="C14:E14" si="2">SUM(C5:C13)</f>
+        <f t="shared" ref="C14:E14" si="5">SUM(C5:C13)</f>
         <v>1473.8717942959731</v>
       </c>
       <c r="D14" s="22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>1685.4106346098099</v>
       </c>
       <c r="E14" s="23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2156.7417637150811</v>
       </c>
       <c r="F14" s="20">
-        <f t="shared" ref="F14" si="3">SUM(F5:F13)</f>
+        <f t="shared" ref="F14" si="6">SUM(F5:F13)</f>
         <v>1713.9551937343867</v>
       </c>
-    </row>
-    <row r="17" spans="1:26" ht="20.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="H14" s="51">
+        <v>2024</v>
+      </c>
+      <c r="I14" s="62">
+        <v>0.42399999999999999</v>
+      </c>
+      <c r="J14" s="62">
+        <f t="shared" si="3"/>
+        <v>0.15359999999999999</v>
+      </c>
+      <c r="K14" s="38">
+        <v>0.68</v>
+      </c>
+      <c r="L14" s="48">
+        <f t="shared" si="4"/>
+        <v>-0.37647058823529417</v>
+      </c>
+      <c r="N14" s="33">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
+      <c r="I15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" ht="20.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A19" s="31"/>
-      <c r="B19" s="44" t="s">
+      <c r="B19" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="C19" s="44"/>
-      <c r="D19" s="44"/>
-      <c r="E19" s="44"/>
+      <c r="C19" s="56"/>
+      <c r="D19" s="56"/>
+      <c r="E19" s="56"/>
       <c r="F19" s="31"/>
     </row>
-    <row r="20" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A20" s="35" t="s">
         <v>4</v>
       </c>
@@ -1701,7 +1887,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A21" s="32" t="s">
         <v>5</v>
       </c>
@@ -1722,11 +1908,11 @@
         <v>101.16999999999999</v>
       </c>
       <c r="H21" s="2"/>
-      <c r="N21" s="2"/>
-      <c r="T21" s="2"/>
-      <c r="Z21" s="2"/>
-    </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.4">
+      <c r="O21" s="2"/>
+      <c r="U21" s="2"/>
+      <c r="AA21" s="2"/>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A22" s="32" t="s">
         <v>6</v>
       </c>
@@ -1743,11 +1929,11 @@
         <v>176.49799999999999</v>
       </c>
       <c r="F22" s="17">
-        <f t="shared" ref="F22:F29" si="4">AVERAGE(B22:E22)</f>
+        <f t="shared" ref="F22:F29" si="7">AVERAGE(B22:E22)</f>
         <v>113.97375</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A23" s="32" t="s">
         <v>0</v>
       </c>
@@ -1764,11 +1950,11 @@
         <v>577.67599999999993</v>
       </c>
       <c r="F23" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>529.61924999999997</v>
       </c>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A24" s="32" t="s">
         <v>7</v>
       </c>
@@ -1785,11 +1971,11 @@
         <v>26.783999999999999</v>
       </c>
       <c r="F24" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>40.58775</v>
       </c>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A25" s="32" t="s">
         <v>8</v>
       </c>
@@ -1806,11 +1992,11 @@
         <v>110.13000000000001</v>
       </c>
       <c r="F25" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>97.3095</v>
       </c>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A26" s="32" t="s">
         <v>9</v>
       </c>
@@ -1827,11 +2013,11 @@
         <v>53.64</v>
       </c>
       <c r="F26" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>49.459999999999994</v>
       </c>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A27" s="32" t="s">
         <v>10</v>
       </c>
@@ -1848,11 +2034,11 @@
         <v>84.36</v>
       </c>
       <c r="F27" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>77.790000000000006</v>
       </c>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.4">
       <c r="A28" s="32" t="s">
         <v>1</v>
       </c>
@@ -1869,14 +2055,14 @@
         <v>565.12376371508105</v>
       </c>
       <c r="F28" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>329.36019373438671</v>
       </c>
       <c r="G28" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A29" s="33" t="s">
         <v>2</v>
       </c>
@@ -1893,11 +2079,11 @@
         <v>461</v>
       </c>
       <c r="F29" s="17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>363.75</v>
       </c>
     </row>
-    <row r="30" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A30" s="33" t="s">
         <v>19</v>
       </c>
@@ -1906,19 +2092,19 @@
         <v>1530.9765823166829</v>
       </c>
       <c r="C30" s="19">
-        <f t="shared" ref="C30:F30" si="5">SUM(C21:C29)</f>
+        <f t="shared" ref="C30:F30" si="8">SUM(C21:C29)</f>
         <v>1464.2867942959731</v>
       </c>
       <c r="D30" s="19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>1678.66763460981</v>
       </c>
       <c r="E30" s="19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>2138.1507637150808</v>
       </c>
       <c r="F30" s="37">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>1703.0204437343866</v>
       </c>
     </row>
@@ -1934,12 +2120,12 @@
     </row>
     <row r="36" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A36" s="31"/>
-      <c r="B36" s="44" t="s">
+      <c r="B36" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="C36" s="44"/>
-      <c r="D36" s="44"/>
-      <c r="E36" s="44"/>
+      <c r="C36" s="56"/>
+      <c r="D36" s="56"/>
+      <c r="E36" s="56"/>
       <c r="F36" s="31"/>
     </row>
     <row r="37" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
@@ -1971,15 +2157,15 @@
         <v>118.18600000000001</v>
       </c>
       <c r="C38" s="16">
-        <f t="shared" ref="C38:E38" si="6">C67</f>
+        <f t="shared" ref="C38:E38" si="9">C67</f>
         <v>74.753</v>
       </c>
       <c r="D38" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>128.80199999999999</v>
       </c>
       <c r="E38" s="16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>82.938999999999993</v>
       </c>
       <c r="F38" s="17">
@@ -1996,19 +2182,19 @@
         <v>100.309</v>
       </c>
       <c r="C39" s="16">
-        <f t="shared" ref="C39:E39" si="7">C68</f>
+        <f t="shared" ref="C39:E39" si="10">C68</f>
         <v>98.667000000000002</v>
       </c>
       <c r="D39" s="16">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>80.421000000000006</v>
       </c>
       <c r="E39" s="16">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>176.49799999999999</v>
       </c>
       <c r="F39" s="17">
-        <f t="shared" ref="F39:F46" si="8">AVERAGE(B39:E39)</f>
+        <f t="shared" ref="F39:F46" si="11">AVERAGE(B39:E39)</f>
         <v>113.97375</v>
       </c>
     </row>
@@ -2021,19 +2207,19 @@
         <v>551.13499999999999</v>
       </c>
       <c r="C40" s="16">
-        <f t="shared" ref="C40:E40" si="9">C56+C69</f>
+        <f t="shared" ref="C40:E40" si="12">C56+C69</f>
         <v>464.16500000000002</v>
       </c>
       <c r="D40" s="16">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>525.50099999999998</v>
       </c>
       <c r="E40" s="16">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>577.67599999999993</v>
       </c>
       <c r="F40" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>529.61924999999997</v>
       </c>
     </row>
@@ -2046,19 +2232,19 @@
         <v>71.613</v>
       </c>
       <c r="C41" s="16">
-        <f t="shared" ref="C41:E41" si="10">C70</f>
+        <f t="shared" ref="C41:E41" si="13">C70</f>
         <v>36.423000000000002</v>
       </c>
       <c r="D41" s="16">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>27.530999999999999</v>
       </c>
       <c r="E41" s="16">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>26.783999999999999</v>
       </c>
       <c r="F41" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>40.58775</v>
       </c>
     </row>
@@ -2071,19 +2257,19 @@
         <v>89.24</v>
       </c>
       <c r="C42" s="16">
-        <f t="shared" ref="C42:E42" si="11">C71</f>
+        <f t="shared" ref="C42:E42" si="14">C71</f>
         <v>79.738</v>
       </c>
       <c r="D42" s="16">
+        <f t="shared" si="14"/>
+        <v>110.13000000000001</v>
+      </c>
+      <c r="E42" s="16">
+        <f t="shared" si="14"/>
+        <v>110.13000000000001</v>
+      </c>
+      <c r="F42" s="17">
         <f t="shared" si="11"/>
-        <v>110.13000000000001</v>
-      </c>
-      <c r="E42" s="16">
-        <f t="shared" si="11"/>
-        <v>110.13000000000001</v>
-      </c>
-      <c r="F42" s="17">
-        <f t="shared" si="8"/>
         <v>97.3095</v>
       </c>
     </row>
@@ -2096,19 +2282,19 @@
         <v>36.92</v>
       </c>
       <c r="C43" s="16">
-        <f t="shared" ref="C43:E43" si="12">C72</f>
+        <f t="shared" ref="C43:E43" si="15">C72</f>
         <v>53.64</v>
       </c>
       <c r="D43" s="16">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>53.64</v>
       </c>
       <c r="E43" s="16">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>53.64</v>
       </c>
       <c r="F43" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>49.459999999999994</v>
       </c>
     </row>
@@ -2121,19 +2307,19 @@
         <v>58.08</v>
       </c>
       <c r="C44" s="16">
-        <f t="shared" ref="C44:E44" si="13">C73</f>
+        <f t="shared" ref="C44:E44" si="16">C73</f>
         <v>84.36</v>
       </c>
       <c r="D44" s="16">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>84.36</v>
       </c>
       <c r="E44" s="16">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>84.36</v>
       </c>
       <c r="F44" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>77.790000000000006</v>
       </c>
     </row>
@@ -2146,19 +2332,19 @@
         <v>207</v>
       </c>
       <c r="C45" s="16">
-        <f t="shared" ref="C45:E45" si="14">C57</f>
+        <f t="shared" ref="C45:E45" si="17">C57</f>
         <v>239</v>
       </c>
       <c r="D45" s="16">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>175</v>
       </c>
       <c r="E45" s="16">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>175</v>
       </c>
       <c r="F45" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>199</v>
       </c>
       <c r="G45" t="s">
@@ -2174,19 +2360,19 @@
         <v>249</v>
       </c>
       <c r="C46" s="16">
-        <f t="shared" ref="C46:E46" si="15">C58</f>
+        <f t="shared" ref="C46:E46" si="18">C58</f>
         <v>284</v>
       </c>
       <c r="D46" s="16">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>461</v>
       </c>
       <c r="E46" s="16">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>461</v>
       </c>
       <c r="F46" s="17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>363.75</v>
       </c>
     </row>
@@ -2199,19 +2385,19 @@
         <v>1481.4829999999999</v>
       </c>
       <c r="C47" s="22">
-        <f t="shared" ref="C47:F47" si="16">SUM(C38:C46)</f>
+        <f t="shared" ref="C47:F47" si="19">SUM(C38:C46)</f>
         <v>1414.7460000000001</v>
       </c>
       <c r="D47" s="22">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1646.3849999999998</v>
       </c>
       <c r="E47" s="22">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1748.0269999999998</v>
       </c>
       <c r="F47" s="37">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>1572.6602499999999</v>
       </c>
     </row>
@@ -2230,12 +2416,12 @@
     </row>
     <row r="54" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A54" s="25"/>
-      <c r="B54" s="46" t="s">
+      <c r="B54" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="C54" s="47"/>
-      <c r="D54" s="47"/>
-      <c r="E54" s="48"/>
+      <c r="C54" s="59"/>
+      <c r="D54" s="59"/>
+      <c r="E54" s="60"/>
       <c r="F54" s="10"/>
     </row>
     <row r="55" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
@@ -2296,7 +2482,7 @@
         <v>175</v>
       </c>
       <c r="F57" s="28">
-        <f t="shared" ref="F57:F61" si="17">AVERAGE(B57:E57)</f>
+        <f t="shared" ref="F57:F61" si="20">AVERAGE(B57:E57)</f>
         <v>199</v>
       </c>
     </row>
@@ -2317,7 +2503,7 @@
         <v>461</v>
       </c>
       <c r="F58" s="28">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>363.75</v>
       </c>
     </row>
@@ -2330,19 +2516,19 @@
         <v>595</v>
       </c>
       <c r="C59" s="29">
-        <f t="shared" ref="C59:E59" si="18">SUM(C56:C58)</f>
+        <f t="shared" ref="C59:E59" si="21">SUM(C56:C58)</f>
         <v>623</v>
       </c>
       <c r="D59" s="29">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>725</v>
       </c>
       <c r="E59" s="30">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>725</v>
       </c>
       <c r="F59" s="28">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>667</v>
       </c>
     </row>
@@ -2363,7 +2549,7 @@
         <v>836</v>
       </c>
       <c r="F60" s="24">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>891.75</v>
       </c>
     </row>
@@ -2376,19 +2562,19 @@
         <v>1686</v>
       </c>
       <c r="C61" s="38">
-        <f t="shared" ref="C61:E61" si="19">SUM(C59:C60)</f>
+        <f t="shared" ref="C61:E61" si="22">SUM(C59:C60)</f>
         <v>1427</v>
       </c>
       <c r="D61" s="38">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>1561</v>
       </c>
       <c r="E61" s="39">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>1561</v>
       </c>
       <c r="F61" s="24">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>1558.75</v>
       </c>
     </row>
@@ -2404,12 +2590,12 @@
     </row>
     <row r="65" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A65" s="34"/>
-      <c r="B65" s="47" t="s">
+      <c r="B65" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="C65" s="47"/>
-      <c r="D65" s="47"/>
-      <c r="E65" s="47"/>
+      <c r="C65" s="59"/>
+      <c r="D65" s="59"/>
+      <c r="E65" s="59"/>
       <c r="F65" s="34"/>
     </row>
     <row r="66" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
@@ -2470,7 +2656,7 @@
         <v>176.49799999999999</v>
       </c>
       <c r="F68" s="17">
-        <f t="shared" ref="F68:F74" si="20">AVERAGE(B68:E68)</f>
+        <f t="shared" ref="F68:F74" si="23">AVERAGE(B68:E68)</f>
         <v>113.97375</v>
       </c>
     </row>
@@ -2491,7 +2677,7 @@
         <v>488.67599999999999</v>
       </c>
       <c r="F69" s="17">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>425.36924999999997</v>
       </c>
     </row>
@@ -2512,7 +2698,7 @@
         <v>26.783999999999999</v>
       </c>
       <c r="F70" s="17">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>40.58775</v>
       </c>
     </row>
@@ -2533,7 +2719,7 @@
         <v>110.13000000000001</v>
       </c>
       <c r="F71" s="17">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>97.3095</v>
       </c>
     </row>
@@ -2554,7 +2740,7 @@
         <v>53.64</v>
       </c>
       <c r="F72" s="17">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>49.459999999999994</v>
       </c>
     </row>
@@ -2575,7 +2761,7 @@
         <v>84.36</v>
       </c>
       <c r="F73" s="20">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>77.790000000000006</v>
       </c>
     </row>
@@ -2588,19 +2774,19 @@
         <v>886.48299999999995</v>
       </c>
       <c r="C74" s="19">
-        <f t="shared" ref="C74:E74" si="21">SUM(C67:C73)</f>
+        <f t="shared" ref="C74:E74" si="24">SUM(C67:C73)</f>
         <v>791.74600000000009</v>
       </c>
       <c r="D74" s="19">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>921.38499999999999</v>
       </c>
       <c r="E74" s="19">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>1023.027</v>
       </c>
       <c r="F74" s="20">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>905.66025000000002</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update CMM 24-06 working paper and presentation
</commit_message>
<xml_diff>
--- a/2025-MLS-projections/BSIA Catch/2021-2024 BSIA MLS Catch.xlsx
+++ b/2025-MLS-projections/BSIA Catch/2021-2024 BSIA MLS Catch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jon.brodziak\Desktop\2024 WCNPO MLS Rebuilding\2025 MLS projections\BSIA Catch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{393BBA42-5C37-437D-856C-9BAAF57CBFEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E8D0F2D-6FDD-4C5C-89C1-ADBB763BFC7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="326" windowWidth="13766" windowHeight="8185" firstSheet="2" activeTab="3" xr2:uid="{416E3EAD-1861-4C87-937B-DDBEC44D9B39}"/>
+    <workbookView xWindow="377" yWindow="377" windowWidth="13766" windowHeight="8186" firstSheet="2" activeTab="3" xr2:uid="{416E3EAD-1861-4C87-937B-DDBEC44D9B39}"/>
   </bookViews>
   <sheets>
     <sheet name="2021-2024-mls-catch" sheetId="4" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="37">
   <si>
     <t>G3</t>
   </si>
@@ -133,12 +133,6 @@
     <t>From WESTERN AND CENTRAL PACIFIC FISHERIES COMMISSION TUNA FISHERY YEARBOOK 2024</t>
   </si>
   <si>
-    <t>From M. Jussup, Fisheries Research Agency, Japan, 3-Feb-2025</t>
-  </si>
-  <si>
-    <t>Total BSIA for WCNPO MLS Catch Biomass by Fleet Group</t>
-  </si>
-  <si>
     <t>F-Based</t>
   </si>
   <si>
@@ -160,16 +154,22 @@
     <t>F-Based C</t>
   </si>
   <si>
-    <t>Scenario 6</t>
-  </si>
-  <si>
-    <t>Scenario 1</t>
-  </si>
-  <si>
     <t>F-Based 80CI</t>
   </si>
   <si>
     <t>Obs F 80CI</t>
+  </si>
+  <si>
+    <t>From M. Jussup, Fisheries Research Agency, Japan, 26-Feb-2025</t>
+  </si>
+  <si>
+    <t>Scenario 6 from 2024 projections</t>
+  </si>
+  <si>
+    <t>Scenario 1 from 2025 CMM 24-06 projections</t>
+  </si>
+  <si>
+    <t>Total 2025 BSIA for WCNPO MLS Catch Biomass by Fleet Group</t>
   </si>
 </sst>
 </file>
@@ -399,7 +399,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -551,6 +551,21 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -569,19 +584,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1349,7 +1355,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAC168C6-DF10-449B-94B3-ED91F02DF6B4}">
-  <dimension ref="A1:AA74"/>
+  <dimension ref="A1:AA90"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="18.07421875" customWidth="1"/>
@@ -1373,1430 +1379,1471 @@
     <col min="27" max="27" width="7.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="20.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:7" ht="20.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="20.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="49" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="4"/>
-      <c r="B3" s="55" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="5"/>
-      <c r="H3" s="36" t="s">
-        <v>3</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="J3" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="K3" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="L3" s="49" t="s">
-        <v>27</v>
-      </c>
-      <c r="N3" s="36" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="7">
+      <c r="G4" s="36" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A5" s="50">
         <v>2021</v>
       </c>
-      <c r="C4" s="8">
+      <c r="B5" s="45" cm="1">
+        <f t="array" ref="B5:B8">TRANSPOSE(B30:E30)</f>
+        <v>1539.7965823166828</v>
+      </c>
+      <c r="C5" s="29">
+        <v>2970</v>
+      </c>
+      <c r="D5" s="45">
+        <f>G5*1.28</f>
+        <v>614.4</v>
+      </c>
+      <c r="E5" s="46">
+        <f>(B5-C5)/C5</f>
+        <v>-0.48154997228394519</v>
+      </c>
+      <c r="G5" s="32">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A6" s="50">
         <v>2022</v>
       </c>
-      <c r="D4" s="8">
+      <c r="B6" s="45">
+        <v>1473.8717942959731</v>
+      </c>
+      <c r="C6" s="29">
+        <v>3420</v>
+      </c>
+      <c r="D6" s="45">
+        <f t="shared" ref="D6:D8" si="0">G6*1.28</f>
+        <v>729.6</v>
+      </c>
+      <c r="E6" s="46">
+        <f t="shared" ref="E6:E9" si="1">(B6-C6)/C6</f>
+        <v>-0.56904333500117743</v>
+      </c>
+      <c r="G6" s="32">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A7" s="50">
         <v>2023</v>
       </c>
-      <c r="E4" s="9">
-        <v>2024</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="50">
-        <v>2021</v>
-      </c>
-      <c r="I4" s="45" cm="1">
-        <f t="array" ref="I4:I7">TRANSPOSE(B14:E14)</f>
-        <v>1539.7965823166828</v>
-      </c>
-      <c r="J4" s="29">
-        <v>2970</v>
-      </c>
-      <c r="K4" s="45">
-        <f>N4*1.28</f>
-        <v>614.4</v>
-      </c>
-      <c r="L4" s="46">
-        <f>(I4-J4)/J4</f>
-        <v>-0.48154997228394519</v>
-      </c>
-      <c r="N4" s="32">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A5" s="25" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="12">
-        <v>118.18600000000001</v>
-      </c>
-      <c r="C5" s="13">
-        <v>74.753</v>
-      </c>
-      <c r="D5" s="13">
-        <v>128.80199999999999</v>
-      </c>
-      <c r="E5" s="13">
-        <v>82.938999999999993</v>
-      </c>
-      <c r="F5" s="14">
-        <f>AVERAGE(B5:E5)</f>
-        <v>101.16999999999999</v>
-      </c>
-      <c r="H5" s="50">
-        <v>2022</v>
-      </c>
-      <c r="I5" s="45">
-        <v>1473.8717942959731</v>
-      </c>
-      <c r="J5" s="29">
-        <v>3420</v>
-      </c>
-      <c r="K5" s="45">
-        <f t="shared" ref="K5:K7" si="0">N5*1.28</f>
-        <v>729.6</v>
-      </c>
-      <c r="L5" s="46">
-        <f t="shared" ref="L5:L8" si="1">(I5-J5)/J5</f>
-        <v>-0.56904333500117743</v>
-      </c>
-      <c r="N5" s="32">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A6" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="15">
-        <v>100.309</v>
-      </c>
-      <c r="C6" s="16">
-        <v>98.667000000000002</v>
-      </c>
-      <c r="D6" s="16">
-        <v>80.421000000000006</v>
-      </c>
-      <c r="E6" s="16">
-        <v>176.49799999999999</v>
-      </c>
-      <c r="F6" s="17">
-        <f t="shared" ref="F6:F13" si="2">AVERAGE(B6:E6)</f>
-        <v>113.97375</v>
-      </c>
-      <c r="H6" s="50">
-        <v>2023</v>
-      </c>
-      <c r="I6" s="45">
+      <c r="B7" s="45">
         <v>1685.4106346098099</v>
       </c>
-      <c r="J6" s="29">
+      <c r="C7" s="29">
         <v>3380</v>
       </c>
-      <c r="K6" s="45">
+      <c r="D7" s="45">
         <f t="shared" si="0"/>
         <v>857.6</v>
       </c>
-      <c r="L6" s="46">
+      <c r="E7" s="46">
         <f t="shared" si="1"/>
         <v>-0.50135780041129885</v>
       </c>
-      <c r="N6" s="32">
+      <c r="G7" s="32">
         <v>670</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" s="15">
-        <v>551.13499999999999</v>
-      </c>
-      <c r="C7" s="16">
-        <v>464.16500000000002</v>
-      </c>
-      <c r="D7" s="16">
-        <v>525.50099999999998</v>
-      </c>
-      <c r="E7" s="16">
-        <v>577.67599999999993</v>
-      </c>
-      <c r="F7" s="17">
-        <f t="shared" si="2"/>
-        <v>529.61924999999997</v>
-      </c>
-      <c r="H7" s="51">
+    <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="51">
         <v>2024</v>
       </c>
-      <c r="I7" s="47">
+      <c r="B8" s="47">
         <v>2156.7417637150811</v>
       </c>
-      <c r="J7" s="38">
+      <c r="C8" s="38">
         <v>3080</v>
       </c>
-      <c r="K7" s="45">
+      <c r="D8" s="45">
         <f t="shared" si="0"/>
         <v>896</v>
       </c>
-      <c r="L7" s="48">
+      <c r="E8" s="48">
         <f t="shared" si="1"/>
         <v>-0.29975916762497368</v>
       </c>
-      <c r="N7" s="33">
+      <c r="G8" s="33">
         <v>700</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="15">
-        <v>71.613</v>
-      </c>
-      <c r="C8" s="16">
-        <v>36.423000000000002</v>
-      </c>
-      <c r="D8" s="16">
-        <v>27.530999999999999</v>
-      </c>
-      <c r="E8" s="16">
-        <v>26.783999999999999</v>
-      </c>
-      <c r="F8" s="17">
-        <f t="shared" si="2"/>
-        <v>40.58775</v>
-      </c>
-      <c r="H8" s="36" t="s">
+    <row r="9" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="52">
-        <f>SUM(_xlfn.ANCHORARRAY(I4))</f>
+      <c r="B9" s="52">
+        <f>SUM(_xlfn.ANCHORARRAY(B5))</f>
         <v>6855.820774937547</v>
       </c>
-      <c r="J8" s="53">
-        <f>SUM(J4:J7)</f>
+      <c r="C9" s="53">
+        <f>SUM(C5:C8)</f>
         <v>12850</v>
       </c>
-      <c r="K8" s="53" t="s">
-        <v>33</v>
-      </c>
-      <c r="L8" s="54">
+      <c r="D9" s="53"/>
+      <c r="E9" s="54">
         <f t="shared" si="1"/>
         <v>-0.46647309144454885</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="26" t="s">
+    <row r="10" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="43" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="49" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="36" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A12" s="57">
+        <v>2021</v>
+      </c>
+      <c r="B12" s="58">
+        <v>0.52700000000000002</v>
+      </c>
+      <c r="C12" s="58">
+        <f>1.28*G12</f>
+        <v>0.1216</v>
+      </c>
+      <c r="D12" s="44">
+        <v>0.68</v>
+      </c>
+      <c r="E12" s="59">
+        <f>(B12-D12)/D12</f>
+        <v>-0.22500000000000003</v>
+      </c>
+      <c r="G12" s="32">
+        <v>9.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A13" s="50">
+        <v>2022</v>
+      </c>
+      <c r="B13" s="55">
+        <v>0.373</v>
+      </c>
+      <c r="C13" s="55">
+        <f t="shared" ref="C13:C15" si="2">1.28*G13</f>
+        <v>9.6000000000000002E-2</v>
+      </c>
+      <c r="D13" s="29">
+        <v>0.68</v>
+      </c>
+      <c r="E13" s="46">
+        <f t="shared" ref="E13:E15" si="3">(B13-D13)/D13</f>
+        <v>-0.45147058823529418</v>
+      </c>
+      <c r="G13" s="32">
+        <v>7.4999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A14" s="50">
+        <v>2023</v>
+      </c>
+      <c r="B14" s="55">
+        <v>0.38100000000000001</v>
+      </c>
+      <c r="C14" s="55">
+        <f t="shared" si="2"/>
+        <v>0.11648</v>
+      </c>
+      <c r="D14" s="29">
+        <v>0.68</v>
+      </c>
+      <c r="E14" s="46">
+        <f t="shared" si="3"/>
+        <v>-0.43970588235294122</v>
+      </c>
+      <c r="G14" s="32">
+        <v>9.0999999999999998E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="51">
+        <v>2024</v>
+      </c>
+      <c r="B15" s="56">
+        <v>0.42399999999999999</v>
+      </c>
+      <c r="C15" s="56">
+        <f t="shared" si="2"/>
+        <v>0.15359999999999999</v>
+      </c>
+      <c r="D15" s="38">
+        <v>0.68</v>
+      </c>
+      <c r="E15" s="48">
+        <f t="shared" si="3"/>
+        <v>-0.37647058823529417</v>
+      </c>
+      <c r="G15" s="33">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A16" s="66"/>
+      <c r="B16" s="55"/>
+      <c r="C16" s="55"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="67"/>
+      <c r="G16" s="29"/>
+    </row>
+    <row r="17" spans="1:6" ht="20.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="4"/>
+      <c r="B19" s="60" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" s="61"/>
+      <c r="D19" s="61"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="5"/>
+    </row>
+    <row r="20" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" s="7">
+        <v>2021</v>
+      </c>
+      <c r="C20" s="8">
+        <v>2022</v>
+      </c>
+      <c r="D20" s="8">
+        <v>2023</v>
+      </c>
+      <c r="E20" s="9">
+        <v>2024</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A21" s="25" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="12">
+        <v>118.18600000000001</v>
+      </c>
+      <c r="C21" s="13">
+        <v>74.753</v>
+      </c>
+      <c r="D21" s="13">
+        <v>128.80199999999999</v>
+      </c>
+      <c r="E21" s="13">
+        <v>82.938999999999993</v>
+      </c>
+      <c r="F21" s="14">
+        <f>AVERAGE(B21:E21)</f>
+        <v>101.16999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A22" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" s="15">
+        <v>100.309</v>
+      </c>
+      <c r="C22" s="16">
+        <v>98.667000000000002</v>
+      </c>
+      <c r="D22" s="16">
+        <v>80.421000000000006</v>
+      </c>
+      <c r="E22" s="16">
+        <v>176.49799999999999</v>
+      </c>
+      <c r="F22" s="17">
+        <f t="shared" ref="F22:F29" si="4">AVERAGE(B22:E22)</f>
+        <v>113.97375</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A23" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B23" s="15">
+        <v>551.13499999999999</v>
+      </c>
+      <c r="C23" s="16">
+        <v>464.16500000000002</v>
+      </c>
+      <c r="D23" s="16">
+        <v>525.50099999999998</v>
+      </c>
+      <c r="E23" s="16">
+        <v>577.67599999999993</v>
+      </c>
+      <c r="F23" s="17">
+        <f t="shared" si="4"/>
+        <v>529.61924999999997</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A24" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="15">
+        <v>71.613</v>
+      </c>
+      <c r="C24" s="16">
+        <v>36.423000000000002</v>
+      </c>
+      <c r="D24" s="16">
+        <v>27.530999999999999</v>
+      </c>
+      <c r="E24" s="16">
+        <v>26.783999999999999</v>
+      </c>
+      <c r="F24" s="17">
+        <f t="shared" si="4"/>
+        <v>40.58775</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A25" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="15">
+      <c r="B25" s="15">
         <v>89.24</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C25" s="16">
         <v>79.738</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D25" s="16">
         <v>110.13000000000001</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E25" s="16">
         <v>110.13000000000001</v>
       </c>
-      <c r="F9" s="17">
-        <f t="shared" si="2"/>
+      <c r="F25" s="17">
+        <f t="shared" si="4"/>
         <v>97.3095</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="26" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A26" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B26" s="15">
         <v>36.92</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C26" s="16">
         <v>53.64</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D26" s="16">
         <v>53.64</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E26" s="16">
         <v>53.64</v>
       </c>
-      <c r="F10" s="17">
-        <f t="shared" si="2"/>
+      <c r="F26" s="17">
+        <f t="shared" si="4"/>
         <v>49.459999999999994</v>
       </c>
-      <c r="H10" s="36" t="s">
-        <v>3</v>
-      </c>
-      <c r="I10" s="43" t="s">
-        <v>30</v>
-      </c>
-      <c r="J10" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="K10" s="43" t="s">
-        <v>26</v>
-      </c>
-      <c r="L10" s="49" t="s">
-        <v>27</v>
-      </c>
-      <c r="N10" s="36" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A11" s="26" t="s">
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A27" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B27" s="15">
         <v>58.08</v>
       </c>
-      <c r="C11" s="16">
+      <c r="C27" s="16">
         <v>84.36</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D27" s="16">
         <v>84.36</v>
       </c>
-      <c r="E11" s="16">
+      <c r="E27" s="16">
         <v>84.36</v>
       </c>
-      <c r="F11" s="17">
-        <f t="shared" si="2"/>
+      <c r="F27" s="17">
+        <f t="shared" si="4"/>
         <v>77.790000000000006</v>
       </c>
-      <c r="H11" s="63">
-        <v>2021</v>
-      </c>
-      <c r="I11" s="64">
-        <v>0.52700000000000002</v>
-      </c>
-      <c r="J11" s="64">
-        <f>1.28*N11</f>
-        <v>0.1216</v>
-      </c>
-      <c r="K11" s="44">
-        <v>0.68</v>
-      </c>
-      <c r="L11" s="65">
-        <f>(I11-K11)/K11</f>
-        <v>-0.22500000000000003</v>
-      </c>
-      <c r="N11" s="32">
-        <v>9.5000000000000001E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="A12" s="26" t="s">
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A28" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B28" s="15">
         <v>265.31358231668298</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C28" s="16">
         <v>298.12579429597298</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D28" s="16">
         <v>214.02563460981</v>
       </c>
-      <c r="E12" s="16">
+      <c r="E28" s="16">
         <v>583.71476371508106</v>
       </c>
-      <c r="F12" s="17">
-        <f t="shared" si="2"/>
+      <c r="F28" s="17">
+        <f t="shared" si="4"/>
         <v>340.29494373438672</v>
       </c>
-      <c r="H12" s="50">
-        <v>2022</v>
-      </c>
-      <c r="I12" s="61">
-        <v>0.373</v>
-      </c>
-      <c r="J12" s="61">
-        <f t="shared" ref="J12:J14" si="3">1.28*N12</f>
-        <v>9.6000000000000002E-2</v>
-      </c>
-      <c r="K12" s="29">
-        <v>0.68</v>
-      </c>
-      <c r="L12" s="46">
-        <f t="shared" ref="L12:L14" si="4">(I12-K12)/K12</f>
-        <v>-0.45147058823529418</v>
-      </c>
-      <c r="N12" s="32">
-        <v>7.4999999999999997E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="11" t="s">
+    </row>
+    <row r="29" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A29" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B13" s="18">
+      <c r="B29" s="18">
         <v>249</v>
       </c>
-      <c r="C13" s="19">
+      <c r="C29" s="19">
         <v>284</v>
       </c>
-      <c r="D13" s="19">
+      <c r="D29" s="19">
         <v>461</v>
       </c>
-      <c r="E13" s="19">
+      <c r="E29" s="19">
         <v>461</v>
       </c>
-      <c r="F13" s="20">
-        <f t="shared" si="2"/>
+      <c r="F29" s="20">
+        <f t="shared" si="4"/>
         <v>363.75</v>
       </c>
-      <c r="H13" s="50">
-        <v>2023</v>
-      </c>
-      <c r="I13" s="61">
-        <v>0.38100000000000001</v>
-      </c>
-      <c r="J13" s="61">
-        <f t="shared" si="3"/>
-        <v>0.11648</v>
-      </c>
-      <c r="K13" s="29">
-        <v>0.68</v>
-      </c>
-      <c r="L13" s="46">
-        <f t="shared" si="4"/>
-        <v>-0.43970588235294122</v>
-      </c>
-      <c r="N13" s="32">
-        <v>9.0999999999999998E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="11" t="s">
+    </row>
+    <row r="30" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A30" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="21">
-        <f>SUM(B5:B13)</f>
+      <c r="B30" s="21">
+        <f>SUM(B21:B29)</f>
         <v>1539.7965823166828</v>
       </c>
-      <c r="C14" s="22">
-        <f t="shared" ref="C14:E14" si="5">SUM(C5:C13)</f>
+      <c r="C30" s="22">
+        <f t="shared" ref="C30:E30" si="5">SUM(C21:C29)</f>
         <v>1473.8717942959731</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D30" s="22">
         <f t="shared" si="5"/>
         <v>1685.4106346098099</v>
       </c>
-      <c r="E14" s="23">
+      <c r="E30" s="23">
         <f t="shared" si="5"/>
         <v>2156.7417637150811</v>
       </c>
-      <c r="F14" s="20">
-        <f t="shared" ref="F14" si="6">SUM(F5:F13)</f>
+      <c r="F30" s="20">
+        <f t="shared" ref="F30" si="6">SUM(F21:F29)</f>
         <v>1713.9551937343867</v>
       </c>
-      <c r="H14" s="51">
+    </row>
+    <row r="33" spans="1:27" ht="20.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A33" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A34" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A35" s="31"/>
+      <c r="B35" s="61" t="s">
+        <v>3</v>
+      </c>
+      <c r="C35" s="61"/>
+      <c r="D35" s="61"/>
+      <c r="E35" s="61"/>
+      <c r="F35" s="31"/>
+    </row>
+    <row r="36" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A36" s="35" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" s="8">
+        <v>2021</v>
+      </c>
+      <c r="C36" s="8">
+        <v>2022</v>
+      </c>
+      <c r="D36" s="8">
+        <v>2023</v>
+      </c>
+      <c r="E36" s="8">
         <v>2024</v>
       </c>
-      <c r="I14" s="62">
-        <v>0.42399999999999999</v>
-      </c>
-      <c r="J14" s="62">
-        <f t="shared" si="3"/>
-        <v>0.15359999999999999</v>
-      </c>
-      <c r="K14" s="38">
-        <v>0.68</v>
-      </c>
-      <c r="L14" s="48">
-        <f t="shared" si="4"/>
-        <v>-0.37647058823529417</v>
-      </c>
-      <c r="N14" s="33">
-        <v>0.12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
-      <c r="I15" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:27" ht="20.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="31"/>
-      <c r="B19" s="56" t="s">
-        <v>3</v>
-      </c>
-      <c r="C19" s="56"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="56"/>
-      <c r="F19" s="31"/>
-    </row>
-    <row r="20" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="35" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20" s="8">
-        <v>2021</v>
-      </c>
-      <c r="C20" s="8">
-        <v>2022</v>
-      </c>
-      <c r="D20" s="8">
-        <v>2023</v>
-      </c>
-      <c r="E20" s="8">
-        <v>2024</v>
-      </c>
-      <c r="F20" s="36" t="s">
+      <c r="F36" s="36" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.4">
-      <c r="A21" s="32" t="s">
+    <row r="37" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A37" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="16">
+      <c r="B37" s="16">
         <v>118.18600000000001</v>
       </c>
-      <c r="C21" s="16">
+      <c r="C37" s="16">
         <v>74.753</v>
       </c>
-      <c r="D21" s="16">
+      <c r="D37" s="16">
         <v>128.80199999999999</v>
       </c>
-      <c r="E21" s="16">
+      <c r="E37" s="16">
         <v>82.938999999999993</v>
       </c>
-      <c r="F21" s="17">
-        <f>AVERAGE(B21:E21)</f>
+      <c r="F37" s="17">
+        <f>AVERAGE(B37:E37)</f>
         <v>101.16999999999999</v>
       </c>
-      <c r="H21" s="2"/>
-      <c r="O21" s="2"/>
-      <c r="U21" s="2"/>
-      <c r="AA21" s="2"/>
-    </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.4">
-      <c r="A22" s="32" t="s">
+      <c r="H37" s="2"/>
+      <c r="O37" s="2"/>
+      <c r="U37" s="2"/>
+      <c r="AA37" s="2"/>
+    </row>
+    <row r="38" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A38" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="16">
+      <c r="B38" s="16">
         <v>100.309</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C38" s="16">
         <v>98.667000000000002</v>
       </c>
-      <c r="D22" s="16">
+      <c r="D38" s="16">
         <v>80.421000000000006</v>
       </c>
-      <c r="E22" s="16">
+      <c r="E38" s="16">
         <v>176.49799999999999</v>
       </c>
-      <c r="F22" s="17">
-        <f t="shared" ref="F22:F29" si="7">AVERAGE(B22:E22)</f>
+      <c r="F38" s="17">
+        <f t="shared" ref="F38:F45" si="7">AVERAGE(B38:E38)</f>
         <v>113.97375</v>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.4">
-      <c r="A23" s="32" t="s">
+    <row r="39" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A39" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B39" s="16">
         <v>551.13499999999999</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C39" s="16">
         <v>464.16500000000002</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D39" s="16">
         <v>525.50099999999998</v>
       </c>
-      <c r="E23" s="16">
+      <c r="E39" s="16">
         <v>577.67599999999993</v>
       </c>
-      <c r="F23" s="17">
+      <c r="F39" s="17">
         <f t="shared" si="7"/>
         <v>529.61924999999997</v>
       </c>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.4">
-      <c r="A24" s="32" t="s">
+    <row r="40" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A40" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B40" s="16">
         <v>71.613</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C40" s="16">
         <v>36.423000000000002</v>
       </c>
-      <c r="D24" s="16">
+      <c r="D40" s="16">
         <v>27.530999999999999</v>
       </c>
-      <c r="E24" s="16">
+      <c r="E40" s="16">
         <v>26.783999999999999</v>
       </c>
-      <c r="F24" s="17">
+      <c r="F40" s="17">
         <f t="shared" si="7"/>
         <v>40.58775</v>
       </c>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.4">
-      <c r="A25" s="32" t="s">
+    <row r="41" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A41" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="16">
+      <c r="B41" s="16">
         <v>89.24</v>
       </c>
-      <c r="C25" s="16">
+      <c r="C41" s="16">
         <v>79.738</v>
       </c>
-      <c r="D25" s="16">
+      <c r="D41" s="16">
         <v>110.13000000000001</v>
       </c>
-      <c r="E25" s="16">
+      <c r="E41" s="16">
         <v>110.13000000000001</v>
       </c>
-      <c r="F25" s="17">
+      <c r="F41" s="17">
         <f t="shared" si="7"/>
         <v>97.3095</v>
       </c>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.4">
-      <c r="A26" s="32" t="s">
+    <row r="42" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A42" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B26" s="16">
+      <c r="B42" s="16">
         <v>36.92</v>
       </c>
-      <c r="C26" s="16">
+      <c r="C42" s="16">
         <v>53.64</v>
       </c>
-      <c r="D26" s="16">
+      <c r="D42" s="16">
         <v>53.64</v>
       </c>
-      <c r="E26" s="16">
+      <c r="E42" s="16">
         <v>53.64</v>
       </c>
-      <c r="F26" s="17">
+      <c r="F42" s="17">
         <f t="shared" si="7"/>
         <v>49.459999999999994</v>
       </c>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.4">
-      <c r="A27" s="32" t="s">
+    <row r="43" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A43" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B27" s="16">
+      <c r="B43" s="16">
         <v>58.08</v>
       </c>
-      <c r="C27" s="16">
+      <c r="C43" s="16">
         <v>84.36</v>
       </c>
-      <c r="D27" s="16">
+      <c r="D43" s="16">
         <v>84.36</v>
       </c>
-      <c r="E27" s="16">
+      <c r="E43" s="16">
         <v>84.36</v>
       </c>
-      <c r="F27" s="17">
+      <c r="F43" s="17">
         <f t="shared" si="7"/>
         <v>77.790000000000006</v>
       </c>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.4">
-      <c r="A28" s="32" t="s">
+    <row r="44" spans="1:27" x14ac:dyDescent="0.4">
+      <c r="A44" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B28" s="16">
+      <c r="B44" s="16">
         <v>256.49358231668299</v>
       </c>
-      <c r="C28" s="16">
+      <c r="C44" s="16">
         <v>288.540794295973</v>
       </c>
-      <c r="D28" s="16">
+      <c r="D44" s="16">
         <v>207.28263460981</v>
       </c>
-      <c r="E28" s="16">
+      <c r="E44" s="16">
         <v>565.12376371508105</v>
       </c>
-      <c r="F28" s="17">
+      <c r="F44" s="17">
         <f t="shared" si="7"/>
         <v>329.36019373438671</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G44" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="33" t="s">
+    <row r="45" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A45" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="B29" s="19">
+      <c r="B45" s="19">
         <v>249</v>
       </c>
-      <c r="C29" s="19">
+      <c r="C45" s="19">
         <v>284</v>
       </c>
-      <c r="D29" s="19">
+      <c r="D45" s="19">
         <v>461</v>
       </c>
-      <c r="E29" s="19">
+      <c r="E45" s="19">
         <v>461</v>
       </c>
-      <c r="F29" s="17">
+      <c r="F45" s="17">
         <f t="shared" si="7"/>
         <v>363.75</v>
       </c>
     </row>
-    <row r="30" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="33" t="s">
+    <row r="46" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A46" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="19">
-        <f>SUM(B21:B29)</f>
+      <c r="B46" s="19">
+        <f>SUM(B37:B45)</f>
         <v>1530.9765823166829</v>
       </c>
-      <c r="C30" s="19">
-        <f t="shared" ref="C30:F30" si="8">SUM(C21:C29)</f>
+      <c r="C46" s="19">
+        <f t="shared" ref="C46:F46" si="8">SUM(C37:C45)</f>
         <v>1464.2867942959731</v>
       </c>
-      <c r="D30" s="19">
+      <c r="D46" s="19">
         <f t="shared" si="8"/>
         <v>1678.66763460981</v>
       </c>
-      <c r="E30" s="19">
+      <c r="E46" s="19">
         <f t="shared" si="8"/>
         <v>2138.1507637150808</v>
       </c>
-      <c r="F30" s="37">
+      <c r="F46" s="37">
         <f t="shared" si="8"/>
         <v>1703.0204437343866</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="20.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="1" t="s">
+    <row r="50" spans="1:7" ht="20.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A50" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
+    <row r="51" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A51" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="31"/>
-      <c r="B36" s="56" t="s">
+    <row r="52" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A52" s="31"/>
+      <c r="B52" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="C36" s="56"/>
-      <c r="D36" s="56"/>
-      <c r="E36" s="56"/>
-      <c r="F36" s="31"/>
-    </row>
-    <row r="37" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="35" t="s">
+      <c r="C52" s="61"/>
+      <c r="D52" s="61"/>
+      <c r="E52" s="61"/>
+      <c r="F52" s="31"/>
+    </row>
+    <row r="53" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A53" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B53" s="8">
         <v>2021</v>
       </c>
-      <c r="C37" s="8">
+      <c r="C53" s="8">
         <v>2022</v>
       </c>
-      <c r="D37" s="8">
+      <c r="D53" s="8">
         <v>2023</v>
       </c>
-      <c r="E37" s="8">
+      <c r="E53" s="8">
         <v>2024</v>
       </c>
-      <c r="F37" s="36" t="s">
+      <c r="F53" s="36" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A38" s="32" t="s">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A54" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B38" s="16">
-        <f>B67</f>
+      <c r="B54" s="16">
+        <f>B83</f>
         <v>118.18600000000001</v>
       </c>
-      <c r="C38" s="16">
-        <f t="shared" ref="C38:E38" si="9">C67</f>
+      <c r="C54" s="16">
+        <f t="shared" ref="C54:E54" si="9">C83</f>
         <v>74.753</v>
       </c>
-      <c r="D38" s="16">
+      <c r="D54" s="16">
         <f t="shared" si="9"/>
         <v>128.80199999999999</v>
       </c>
-      <c r="E38" s="16">
+      <c r="E54" s="16">
         <f t="shared" si="9"/>
         <v>82.938999999999993</v>
       </c>
-      <c r="F38" s="17">
-        <f>AVERAGE(B38:E38)</f>
+      <c r="F54" s="17">
+        <f>AVERAGE(B54:E54)</f>
         <v>101.16999999999999</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A39" s="32" t="s">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A55" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B39" s="16">
-        <f>B68</f>
+      <c r="B55" s="16">
+        <f>B84</f>
         <v>100.309</v>
       </c>
-      <c r="C39" s="16">
-        <f t="shared" ref="C39:E39" si="10">C68</f>
+      <c r="C55" s="16">
+        <f t="shared" ref="C55:E55" si="10">C84</f>
         <v>98.667000000000002</v>
       </c>
-      <c r="D39" s="16">
+      <c r="D55" s="16">
         <f t="shared" si="10"/>
         <v>80.421000000000006</v>
       </c>
-      <c r="E39" s="16">
+      <c r="E55" s="16">
         <f t="shared" si="10"/>
         <v>176.49799999999999</v>
       </c>
-      <c r="F39" s="17">
-        <f t="shared" ref="F39:F46" si="11">AVERAGE(B39:E39)</f>
+      <c r="F55" s="17">
+        <f t="shared" ref="F55:F62" si="11">AVERAGE(B55:E55)</f>
         <v>113.97375</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A40" s="32" t="s">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A56" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B40" s="16">
-        <f>B56+B69</f>
+      <c r="B56" s="16">
+        <f>B72+B85</f>
         <v>551.13499999999999</v>
       </c>
-      <c r="C40" s="16">
-        <f t="shared" ref="C40:E40" si="12">C56+C69</f>
+      <c r="C56" s="16">
+        <f t="shared" ref="C56:E56" si="12">C72+C85</f>
         <v>464.16500000000002</v>
       </c>
-      <c r="D40" s="16">
+      <c r="D56" s="16">
         <f t="shared" si="12"/>
         <v>525.50099999999998</v>
       </c>
-      <c r="E40" s="16">
+      <c r="E56" s="16">
         <f t="shared" si="12"/>
         <v>577.67599999999993</v>
       </c>
-      <c r="F40" s="17">
+      <c r="F56" s="17">
         <f t="shared" si="11"/>
         <v>529.61924999999997</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A41" s="32" t="s">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A57" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="B41" s="16">
-        <f>B70</f>
+      <c r="B57" s="16">
+        <f>B86</f>
         <v>71.613</v>
       </c>
-      <c r="C41" s="16">
-        <f t="shared" ref="C41:E41" si="13">C70</f>
+      <c r="C57" s="16">
+        <f t="shared" ref="C57:E57" si="13">C86</f>
         <v>36.423000000000002</v>
       </c>
-      <c r="D41" s="16">
+      <c r="D57" s="16">
         <f t="shared" si="13"/>
         <v>27.530999999999999</v>
       </c>
-      <c r="E41" s="16">
+      <c r="E57" s="16">
         <f t="shared" si="13"/>
         <v>26.783999999999999</v>
       </c>
-      <c r="F41" s="17">
+      <c r="F57" s="17">
         <f t="shared" si="11"/>
         <v>40.58775</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A42" s="32" t="s">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A58" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="B42" s="16">
-        <f>B71</f>
+      <c r="B58" s="16">
+        <f>B87</f>
         <v>89.24</v>
       </c>
-      <c r="C42" s="16">
-        <f t="shared" ref="C42:E42" si="14">C71</f>
+      <c r="C58" s="16">
+        <f t="shared" ref="C58:E58" si="14">C87</f>
         <v>79.738</v>
       </c>
-      <c r="D42" s="16">
+      <c r="D58" s="16">
         <f t="shared" si="14"/>
         <v>110.13000000000001</v>
       </c>
-      <c r="E42" s="16">
+      <c r="E58" s="16">
         <f t="shared" si="14"/>
         <v>110.13000000000001</v>
       </c>
-      <c r="F42" s="17">
+      <c r="F58" s="17">
         <f t="shared" si="11"/>
         <v>97.3095</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A43" s="32" t="s">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A59" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B43" s="16">
-        <f>B72</f>
+      <c r="B59" s="16">
+        <f>B88</f>
         <v>36.92</v>
       </c>
-      <c r="C43" s="16">
-        <f t="shared" ref="C43:E43" si="15">C72</f>
+      <c r="C59" s="16">
+        <f t="shared" ref="C59:E59" si="15">C88</f>
         <v>53.64</v>
       </c>
-      <c r="D43" s="16">
+      <c r="D59" s="16">
         <f t="shared" si="15"/>
         <v>53.64</v>
       </c>
-      <c r="E43" s="16">
+      <c r="E59" s="16">
         <f t="shared" si="15"/>
         <v>53.64</v>
       </c>
-      <c r="F43" s="17">
+      <c r="F59" s="17">
         <f t="shared" si="11"/>
         <v>49.459999999999994</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A44" s="32" t="s">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A60" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B44" s="16">
-        <f>B73</f>
+      <c r="B60" s="16">
+        <f>B89</f>
         <v>58.08</v>
       </c>
-      <c r="C44" s="16">
-        <f t="shared" ref="C44:E44" si="16">C73</f>
+      <c r="C60" s="16">
+        <f t="shared" ref="C60:E60" si="16">C89</f>
         <v>84.36</v>
       </c>
-      <c r="D44" s="16">
+      <c r="D60" s="16">
         <f t="shared" si="16"/>
         <v>84.36</v>
       </c>
-      <c r="E44" s="16">
+      <c r="E60" s="16">
         <f t="shared" si="16"/>
         <v>84.36</v>
       </c>
-      <c r="F44" s="17">
+      <c r="F60" s="17">
         <f t="shared" si="11"/>
         <v>77.790000000000006</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A45" s="32" t="s">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A61" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B45" s="16">
-        <f>B57</f>
+      <c r="B61" s="16">
+        <f>B73</f>
         <v>207</v>
       </c>
-      <c r="C45" s="16">
-        <f t="shared" ref="C45:E45" si="17">C57</f>
+      <c r="C61" s="16">
+        <f t="shared" ref="C61:E61" si="17">C73</f>
         <v>239</v>
       </c>
-      <c r="D45" s="16">
+      <c r="D61" s="16">
         <f t="shared" si="17"/>
         <v>175</v>
       </c>
-      <c r="E45" s="16">
+      <c r="E61" s="16">
         <f t="shared" si="17"/>
         <v>175</v>
       </c>
-      <c r="F45" s="17">
+      <c r="F61" s="17">
         <f t="shared" si="11"/>
         <v>199</v>
       </c>
-      <c r="G45" t="s">
+      <c r="G61" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A46" s="32" t="s">
+    <row r="62" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A62" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B46" s="16">
-        <f>B58</f>
+      <c r="B62" s="16">
+        <f>B74</f>
         <v>249</v>
       </c>
-      <c r="C46" s="16">
-        <f t="shared" ref="C46:E46" si="18">C58</f>
+      <c r="C62" s="16">
+        <f t="shared" ref="C62:E62" si="18">C74</f>
         <v>284</v>
       </c>
-      <c r="D46" s="16">
+      <c r="D62" s="16">
         <f t="shared" si="18"/>
         <v>461</v>
       </c>
-      <c r="E46" s="16">
+      <c r="E62" s="16">
         <f t="shared" si="18"/>
         <v>461</v>
       </c>
-      <c r="F46" s="17">
+      <c r="F62" s="17">
         <f t="shared" si="11"/>
         <v>363.75</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="36" t="s">
+    <row r="63" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A63" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="22">
-        <f>SUM(B38:B46)</f>
+      <c r="B63" s="22">
+        <f>SUM(B54:B62)</f>
         <v>1481.4829999999999</v>
       </c>
-      <c r="C47" s="22">
-        <f t="shared" ref="C47:F47" si="19">SUM(C38:C46)</f>
+      <c r="C63" s="22">
+        <f t="shared" ref="C63:F63" si="19">SUM(C54:C62)</f>
         <v>1414.7460000000001</v>
       </c>
-      <c r="D47" s="22">
+      <c r="D63" s="22">
         <f t="shared" si="19"/>
         <v>1646.3849999999998</v>
       </c>
-      <c r="E47" s="22">
+      <c r="E63" s="22">
         <f t="shared" si="19"/>
         <v>1748.0269999999998</v>
       </c>
-      <c r="F47" s="37">
+      <c r="F63" s="37">
         <f t="shared" si="19"/>
         <v>1572.6602499999999</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="F50" s="3"/>
-    </row>
-    <row r="52" spans="1:6" ht="26.15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A52" s="1" t="s">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="F66" s="3"/>
+    </row>
+    <row r="68" spans="1:6" ht="26.15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A68" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A53" s="42" t="s">
+    <row r="69" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A69" s="42" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A54" s="25"/>
-      <c r="B54" s="58" t="s">
+    <row r="70" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A70" s="25"/>
+      <c r="B70" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C54" s="59"/>
-      <c r="D54" s="59"/>
-      <c r="E54" s="60"/>
-      <c r="F54" s="10"/>
-    </row>
-    <row r="55" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A55" s="41" t="s">
+      <c r="C70" s="64"/>
+      <c r="D70" s="64"/>
+      <c r="E70" s="65"/>
+      <c r="F70" s="10"/>
+    </row>
+    <row r="71" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A71" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="B55" s="7">
+      <c r="B71" s="7">
         <v>2021</v>
       </c>
-      <c r="C55" s="8">
+      <c r="C71" s="8">
         <v>2022</v>
       </c>
-      <c r="D55" s="8">
+      <c r="D71" s="8">
         <v>2023</v>
       </c>
-      <c r="E55" s="9">
+      <c r="E71" s="9">
         <v>2024</v>
       </c>
-      <c r="F55" s="9" t="s">
+      <c r="F71" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A56" s="25" t="s">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A72" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B56" s="25">
+      <c r="B72" s="25">
         <v>139</v>
       </c>
-      <c r="C56" s="27">
+      <c r="C72" s="27">
         <v>100</v>
       </c>
-      <c r="D56" s="27">
+      <c r="D72" s="27">
         <v>89</v>
       </c>
-      <c r="E56" s="10">
+      <c r="E72" s="10">
         <v>89</v>
       </c>
-      <c r="F56" s="40">
-        <f>AVERAGE(B56:E56)</f>
+      <c r="F72" s="40">
+        <f>AVERAGE(B72:E72)</f>
         <v>104.25</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A57" s="26" t="s">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A73" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B57" s="26">
+      <c r="B73" s="26">
         <v>207</v>
       </c>
-      <c r="C57" s="29">
+      <c r="C73" s="29">
         <v>239</v>
       </c>
-      <c r="D57" s="29">
+      <c r="D73" s="29">
         <v>175</v>
       </c>
-      <c r="E57" s="30">
+      <c r="E73" s="30">
         <v>175</v>
       </c>
-      <c r="F57" s="28">
-        <f t="shared" ref="F57:F61" si="20">AVERAGE(B57:E57)</f>
+      <c r="F73" s="28">
+        <f t="shared" ref="F73:F77" si="20">AVERAGE(B73:E73)</f>
         <v>199</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A58" s="26" t="s">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A74" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="B58" s="26">
+      <c r="B74" s="26">
         <v>249</v>
       </c>
-      <c r="C58" s="29">
+      <c r="C74" s="29">
         <v>284</v>
       </c>
-      <c r="D58" s="29">
+      <c r="D74" s="29">
         <v>461</v>
       </c>
-      <c r="E58" s="30">
+      <c r="E74" s="30">
         <v>461</v>
       </c>
-      <c r="F58" s="28">
+      <c r="F74" s="28">
         <f t="shared" si="20"/>
         <v>363.75</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A59" s="26" t="s">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A75" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B59" s="26">
-        <f>SUM(B56:B58)</f>
+      <c r="B75" s="26">
+        <f>SUM(B72:B74)</f>
         <v>595</v>
       </c>
-      <c r="C59" s="29">
-        <f t="shared" ref="C59:E59" si="21">SUM(C56:C58)</f>
+      <c r="C75" s="29">
+        <f t="shared" ref="C75:E75" si="21">SUM(C72:C74)</f>
         <v>623</v>
       </c>
-      <c r="D59" s="29">
+      <c r="D75" s="29">
         <f t="shared" si="21"/>
         <v>725</v>
       </c>
-      <c r="E59" s="30">
+      <c r="E75" s="30">
         <f t="shared" si="21"/>
         <v>725</v>
       </c>
-      <c r="F59" s="28">
+      <c r="F75" s="28">
         <f t="shared" si="20"/>
         <v>667</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A60" s="11" t="s">
+    <row r="76" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A76" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B60" s="11">
+      <c r="B76" s="11">
         <v>1091</v>
       </c>
-      <c r="C60" s="38">
+      <c r="C76" s="38">
         <v>804</v>
       </c>
-      <c r="D60" s="38">
+      <c r="D76" s="38">
         <v>836</v>
       </c>
-      <c r="E60" s="39">
+      <c r="E76" s="39">
         <v>836</v>
       </c>
-      <c r="F60" s="24">
+      <c r="F76" s="24">
         <f t="shared" si="20"/>
         <v>891.75</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A61" s="11" t="s">
+    <row r="77" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A77" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B61" s="11">
-        <f>SUM(B59:B60)</f>
+      <c r="B77" s="11">
+        <f>SUM(B75:B76)</f>
         <v>1686</v>
       </c>
-      <c r="C61" s="38">
-        <f t="shared" ref="C61:E61" si="22">SUM(C59:C60)</f>
+      <c r="C77" s="38">
+        <f t="shared" ref="C77:E77" si="22">SUM(C75:C76)</f>
         <v>1427</v>
       </c>
-      <c r="D61" s="38">
+      <c r="D77" s="38">
         <f t="shared" si="22"/>
         <v>1561</v>
       </c>
-      <c r="E61" s="39">
+      <c r="E77" s="39">
         <f t="shared" si="22"/>
         <v>1561</v>
       </c>
-      <c r="F61" s="24">
+      <c r="F77" s="24">
         <f t="shared" si="20"/>
         <v>1558.75</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="20.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A63" s="1" t="s">
+    <row r="79" spans="1:6" ht="20.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A79" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="13.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A64" s="42" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A65" s="34"/>
-      <c r="B65" s="59" t="s">
+    <row r="80" spans="1:6" ht="13.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A80" s="42" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A81" s="34"/>
+      <c r="B81" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="C65" s="59"/>
-      <c r="D65" s="59"/>
-      <c r="E65" s="59"/>
-      <c r="F65" s="34"/>
-    </row>
-    <row r="66" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A66" s="35" t="s">
+      <c r="C81" s="64"/>
+      <c r="D81" s="64"/>
+      <c r="E81" s="64"/>
+      <c r="F81" s="34"/>
+    </row>
+    <row r="82" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A82" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B66" s="8">
+      <c r="B82" s="8">
         <v>2021</v>
       </c>
-      <c r="C66" s="8">
+      <c r="C82" s="8">
         <v>2022</v>
       </c>
-      <c r="D66" s="8">
+      <c r="D82" s="8">
         <v>2023</v>
       </c>
-      <c r="E66" s="8">
+      <c r="E82" s="8">
         <v>2024</v>
       </c>
-      <c r="F66" s="36" t="s">
+      <c r="F82" s="36" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A67" s="32" t="s">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A83" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B67" s="16">
+      <c r="B83" s="16">
         <v>118.18600000000001</v>
       </c>
-      <c r="C67" s="16">
+      <c r="C83" s="16">
         <v>74.753</v>
       </c>
-      <c r="D67" s="16">
+      <c r="D83" s="16">
         <v>128.80199999999999</v>
       </c>
-      <c r="E67" s="16">
+      <c r="E83" s="16">
         <v>82.938999999999993</v>
       </c>
-      <c r="F67" s="17">
-        <f>AVERAGE(B67:E67)</f>
+      <c r="F83" s="17">
+        <f>AVERAGE(B83:E83)</f>
         <v>101.16999999999999</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A68" s="32" t="s">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A84" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B68" s="16">
+      <c r="B84" s="16">
         <v>100.309</v>
       </c>
-      <c r="C68" s="16">
+      <c r="C84" s="16">
         <v>98.667000000000002</v>
       </c>
-      <c r="D68" s="16">
+      <c r="D84" s="16">
         <v>80.421000000000006</v>
       </c>
-      <c r="E68" s="16">
+      <c r="E84" s="16">
         <v>176.49799999999999</v>
       </c>
-      <c r="F68" s="17">
-        <f t="shared" ref="F68:F74" si="23">AVERAGE(B68:E68)</f>
+      <c r="F84" s="17">
+        <f t="shared" ref="F84:F90" si="23">AVERAGE(B84:E84)</f>
         <v>113.97375</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A69" s="32" t="s">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A85" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B69" s="16">
+      <c r="B85" s="16">
         <v>412.13499999999999</v>
       </c>
-      <c r="C69" s="16">
+      <c r="C85" s="16">
         <v>364.16500000000002</v>
       </c>
-      <c r="D69" s="16">
+      <c r="D85" s="16">
         <v>436.50100000000003</v>
       </c>
-      <c r="E69" s="16">
+      <c r="E85" s="16">
         <v>488.67599999999999</v>
       </c>
-      <c r="F69" s="17">
+      <c r="F85" s="17">
         <f t="shared" si="23"/>
         <v>425.36924999999997</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A70" s="32" t="s">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A86" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="B70" s="16">
+      <c r="B86" s="16">
         <v>71.613</v>
       </c>
-      <c r="C70" s="16">
+      <c r="C86" s="16">
         <v>36.423000000000002</v>
       </c>
-      <c r="D70" s="16">
+      <c r="D86" s="16">
         <v>27.530999999999999</v>
       </c>
-      <c r="E70" s="16">
+      <c r="E86" s="16">
         <v>26.783999999999999</v>
       </c>
-      <c r="F70" s="17">
+      <c r="F86" s="17">
         <f t="shared" si="23"/>
         <v>40.58775</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A71" s="32" t="s">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A87" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="B71" s="16">
+      <c r="B87" s="16">
         <v>89.24</v>
       </c>
-      <c r="C71" s="16">
+      <c r="C87" s="16">
         <v>79.738</v>
       </c>
-      <c r="D71" s="16">
+      <c r="D87" s="16">
         <v>110.13000000000001</v>
       </c>
-      <c r="E71" s="16">
+      <c r="E87" s="16">
         <v>110.13000000000001</v>
       </c>
-      <c r="F71" s="17">
+      <c r="F87" s="17">
         <f t="shared" si="23"/>
         <v>97.3095</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A72" s="32" t="s">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A88" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="B72" s="16">
+      <c r="B88" s="16">
         <v>36.92</v>
       </c>
-      <c r="C72" s="16">
+      <c r="C88" s="16">
         <v>53.64</v>
       </c>
-      <c r="D72" s="16">
+      <c r="D88" s="16">
         <v>53.64</v>
       </c>
-      <c r="E72" s="16">
+      <c r="E88" s="16">
         <v>53.64</v>
       </c>
-      <c r="F72" s="17">
+      <c r="F88" s="17">
         <f t="shared" si="23"/>
         <v>49.459999999999994</v>
       </c>
     </row>
-    <row r="73" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A73" s="33" t="s">
+    <row r="89" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A89" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="B73" s="19">
+      <c r="B89" s="19">
         <v>58.08</v>
       </c>
-      <c r="C73" s="19">
+      <c r="C89" s="19">
         <v>84.36</v>
       </c>
-      <c r="D73" s="19">
+      <c r="D89" s="19">
         <v>84.36</v>
       </c>
-      <c r="E73" s="19">
+      <c r="E89" s="19">
         <v>84.36</v>
       </c>
-      <c r="F73" s="20">
+      <c r="F89" s="20">
         <f t="shared" si="23"/>
         <v>77.790000000000006</v>
       </c>
     </row>
-    <row r="74" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A74" s="33" t="s">
+    <row r="90" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A90" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="B74" s="19">
-        <f>SUM(B67:B73)</f>
+      <c r="B90" s="19">
+        <f>SUM(B83:B89)</f>
         <v>886.48299999999995</v>
       </c>
-      <c r="C74" s="19">
-        <f t="shared" ref="C74:E74" si="24">SUM(C67:C73)</f>
+      <c r="C90" s="19">
+        <f t="shared" ref="C90:E90" si="24">SUM(C83:C89)</f>
         <v>791.74600000000009</v>
       </c>
-      <c r="D74" s="19">
+      <c r="D90" s="19">
         <f t="shared" si="24"/>
         <v>921.38499999999999</v>
       </c>
-      <c r="E74" s="19">
+      <c r="E90" s="19">
         <f t="shared" si="24"/>
         <v>1023.027</v>
       </c>
-      <c r="F74" s="20">
+      <c r="F90" s="20">
         <f t="shared" si="23"/>
         <v>905.66025000000002</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="B3:E3"/>
     <mergeCell ref="B19:E19"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="B54:E54"/>
-    <mergeCell ref="B65:E65"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="B70:E70"/>
+    <mergeCell ref="B81:E81"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>